<commit_message>
Add hashtags to captions, humanize copy, add images/ subfolder per post
- Caption Draft column now includes the full hashtag set, copy-paste ready
- Warmer, more personal wording on several captions; no em dashes anywhere
- Every content folder gets an images/ subfolder for final outputs
- Move finished Botox slides into their images/ subfolder

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SLor5oRycb3mTg2nxeqzj7
</commit_message>
<xml_diff>
--- a/strategy/ig-content-strategy.xlsx
+++ b/strategy/ig-content-strategy.xlsx
@@ -207,7 +207,8 @@
     <t xml:space="preserve">5 Botox Lies You Still Believe | The truth, from a nurse injector.</t>
   </si>
   <si>
-    <t xml:space="preserve">Half of what you have heard about Botox came from someone who saw bad work. Let's set the record straight. Which myth did you believe? Drop it below and share this with a friend who needs slide 5. ✨</t>
+    <t xml:space="preserve">Half of what you have heard about Botox came from someone who saw bad work. Let's set the record straight. Which myth did you believe? Drop it below and share this with a friend who needs slide 5. ✨
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">DM BOTOX or link in bio</t>
@@ -237,7 +238,8 @@
     <t xml:space="preserve">Service Spotlight: Botox | Smooth, not frozen.</t>
   </si>
   <si>
-    <t xml:space="preserve">Softened lines, full expression, and nobody can tell why you look so rested. That is Botox done right. ✨</t>
+    <t xml:space="preserve">Softened lines, full expression, and nobody can tell why you look so rested. That is Botox done right. ✨
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">DM BOTOX to book</t>
@@ -261,7 +263,8 @@
     <t xml:space="preserve">5 Red Flags at a Med Spa. Run. | Your face deserves better than a bargain.</t>
   </si>
   <si>
-    <t xml:space="preserve">A menu with no consultation, prices too good to be true, and nobody asking about your medical history. If you see these, walk away. Save this checklist before you book anywhere. 💛</t>
+    <t xml:space="preserve">A menu with no consultation, prices too good to be true, and nobody asking about your medical history. If you see these, walk away. I want you safe, even if you never book with me. Save this checklist. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Save this checklist</t>
@@ -285,7 +288,8 @@
     <t xml:space="preserve">Behind the Scenes: The Prep | Zero shortcuts. Ever.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sealed products, precise dosing, clean everything. This is the part you never see, and the part that matters most. 💛</t>
+    <t xml:space="preserve">Sealed products, precise dosing, clean everything. This is the part you never see, and the part that matters most. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Book with confidence. Link in bio</t>
@@ -303,7 +307,8 @@
     <t xml:space="preserve">Quote: Great Work Is Invisible | Brand quote card.</t>
   </si>
   <si>
-    <t xml:space="preserve">Great work is invisible. Bad work is what gave Botox its reputation. Agree or disagree? 👇</t>
+    <t xml:space="preserve">Great work is invisible. Bad work is what gave Botox its reputation. Agree or disagree? 👇
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Comment below</t>
@@ -318,7 +323,8 @@
     <t xml:space="preserve">Your First Visit, Step by Step | Nervous about your first appointment? Here is exactly what happens.</t>
   </si>
   <si>
-    <t xml:space="preserve">80 percent of first-timers tell me they waited years because they did not know what to expect. Consider this your preview. Send it to the friend who keeps saying one day.</t>
+    <t xml:space="preserve">80 percent of first-timers tell me they waited years because they did not know what to expect. Consider this your preview. Send it to the friend who keeps saying one day.
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Book your consult. Link in bio</t>
@@ -333,7 +339,8 @@
     <t xml:space="preserve">3 Signs Your Injector Is Rushing You | Protect yourself before you book.</t>
   </si>
   <si>
-    <t xml:space="preserve">If your consult is shorter than your coffee order, that is a problem. Save this checklist and trust your gut.</t>
+    <t xml:space="preserve">If your consult is shorter than your coffee order, that is a problem. Save this checklist and trust your gut.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Save + share this</t>
@@ -348,7 +355,8 @@
     <t xml:space="preserve">Meet NP Cleo: The Face Behind the Glow | Real education. Real results. Real care.</t>
   </si>
   <si>
-    <t xml:space="preserve">Before you trust someone with your face, you should know who they are. Here is my story, my training, and why I will always tell you the truth about what you need. 💛</t>
+    <t xml:space="preserve">Before you trust someone with your face, you should know who they are. Here is my story, my training, and why I will always tell you the truth about what you need. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Say hi in the comments</t>
@@ -363,7 +371,8 @@
     <t xml:space="preserve">Welcome to the Treatment Room | Where calm meets careful.</t>
   </si>
   <si>
-    <t xml:space="preserve">Clean, quiet, and designed for you to feel safe asking anything. Come see it in person. 💛</t>
+    <t xml:space="preserve">Clean, quiet, and designed for you to feel safe asking anything. Come see it in person. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Book a visit. Link in bio</t>
@@ -378,7 +387,8 @@
     <t xml:space="preserve">This or That: Rested vs Frozen | Engagement post.</t>
   </si>
   <si>
-    <t xml:space="preserve">When you picture your results, which one are you actually asking for? Vote below. 👇</t>
+    <t xml:space="preserve">When you picture your results, which one are you actually asking for? Vote below. 👇
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Vote in the comments</t>
@@ -393,7 +403,8 @@
     <t xml:space="preserve">Preventative Botox: When to Actually Start | Your friend who never seems to age? This is why.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lines are easier to prevent than to erase. Here is how to know if your late 20s or 30s is the right time to start, and when it is genuinely too early.</t>
+    <t xml:space="preserve">Lines are easier to prevent than to erase. Here is how to know if your late 20s or 30s is the right time to start, and when it is honestly still too early. No pressure, just real timing.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">DM PREVENT for a consult</t>
@@ -411,7 +422,8 @@
     <t xml:space="preserve">Service Spotlight: Preventative Botox | Start before the lines do.</t>
   </si>
   <si>
-    <t xml:space="preserve">The friend who never seems to age did not find a miracle cream. She started early and kept it subtle.</t>
+    <t xml:space="preserve">The friend who never seems to age did not find a miracle cream. She started early and kept it subtle.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">DM PREVENT to talk</t>
@@ -426,7 +438,8 @@
     <t xml:space="preserve">What 20 Units Actually Looks Like | Unit math, finally explained.</t>
   </si>
   <si>
-    <t xml:space="preserve">You have seen the price per unit. But what does 20 units actually do? Here is the honest breakdown of dosing, areas, and why cheaper per unit is not cheaper overall.</t>
+    <t xml:space="preserve">You have seen the price per unit. But what does 20 units actually do? Here is the honest breakdown of dosing, areas, and why cheaper per unit is not cheaper overall.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Save this for your consult</t>
@@ -441,7 +454,8 @@
     <t xml:space="preserve">Meet Your Injector | Board certified. Botox obsessed. Brutally honest.</t>
   </si>
   <si>
-    <t xml:space="preserve">Your face deserves a nurse practitioner who tells the truth about what you need and what you do not. Hi, I am Cleo. 💛</t>
+    <t xml:space="preserve">Your face deserves a nurse practitioner who tells the truth about what you need and what you do not. Hi, I am Cleo. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: Cleo portrait + credentials hook</t>
@@ -453,7 +467,8 @@
     <t xml:space="preserve">Quote: Prevention Beats Erasing | Brand quote card.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lines are easier to prevent than to erase. Save this reminder. ✨</t>
+    <t xml:space="preserve">Lines are easier to prevent than to erase. Save this reminder. ✨
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Save this</t>
@@ -468,7 +483,8 @@
     <t xml:space="preserve">Botox vs Dysport: The Real Difference | Same family. Different personalities.</t>
   </si>
   <si>
-    <t xml:space="preserve">The most Googled question in aesthetics, answered honestly. Slide 5 explains why you should never compare prices unit to unit. Save this for later. ✨</t>
+    <t xml:space="preserve">The most Googled question in aesthetics, answered honestly. Slide 5 explains why you should never compare prices unit to unit. Save this for later. ✨
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Book a consult. Link in bio</t>
@@ -480,7 +496,8 @@
     <t xml:space="preserve">Botox vs Dysport at a Glance | Same family. Different personalities.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dysport kicks in faster and spreads wider. Botox is precise. The right one depends on your face, not the price list.</t>
+    <t xml:space="preserve">Dysport kicks in faster and spreads wider. Botox is precise. The right one depends on your face, not the price list.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Full breakdown on our feed</t>
@@ -495,7 +512,8 @@
     <t xml:space="preserve">Botox Aftercare: The First 48 Hours | You got Botox. Now what?</t>
   </si>
   <si>
-    <t xml:space="preserve">The first 48 hours matter more than most people think. Here is exactly what to do, what to skip, and when to call me. Bookmark this one.</t>
+    <t xml:space="preserve">The first 48 hours matter more than most people think. Here is exactly what to do, what to skip, and when to call me. Bookmark this one.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Save this guide</t>
@@ -507,7 +525,8 @@
     <t xml:space="preserve">The Face Map | Every face gets a plan.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nothing touches your skin before I map your anatomy, your movement, and your goals. Planning is the treatment.</t>
+    <t xml:space="preserve">Nothing touches your skin before I map your anatomy, your movement, and your goals. Planning is the treatment.
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Book your mapping. Link in bio</t>
@@ -522,7 +541,8 @@
     <t xml:space="preserve">FAQ: Does Botox Hurt? | Honest answer, no fluff.</t>
   </si>
   <si>
-    <t xml:space="preserve">The honest answer: less than plucking a brow. Tiny needle, seconds per area, numbing if you want it.</t>
+    <t xml:space="preserve">Honestly? Less than plucking a brow. Tiny needle, a few seconds per area, and numbing if you want it. Most people say wait, that was it?
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">More questions? DM me</t>
@@ -537,7 +557,8 @@
     <t xml:space="preserve">5 Things Botox Can't Do | Honest expectations, always.</t>
   </si>
   <si>
-    <t xml:space="preserve">Botox is amazing at what it does. But it cannot do everything, and anyone who says otherwise is selling you something. Here is what it fixes and what needs a different plan.</t>
+    <t xml:space="preserve">Botox is amazing at what it does. But it cannot do everything, and anyone who says otherwise is selling you something. Here is what it fixes and what needs a different plan.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Comment your questions</t>
@@ -549,7 +570,8 @@
     <t xml:space="preserve">What Botox Can't Fix | Honest expectations, always.</t>
   </si>
   <si>
-    <t xml:space="preserve">Sagging skin, volume loss, texture. Botox is not the tool for everything, and I will always tell you what is.</t>
+    <t xml:space="preserve">Sagging skin, volume loss, texture. Botox is not the tool for everything, and I would rather tell you that now than take your money and disappoint you.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: myth-vs-reality card</t>
@@ -561,7 +583,8 @@
     <t xml:space="preserve">Still You, Just Refreshed | You won't look done. You'll look rested.</t>
   </si>
   <si>
-    <t xml:space="preserve">The 2026 standard is not transformation. It is restoration. My goal is that people ask if you have been on vacation, not what you had done. 💛</t>
+    <t xml:space="preserve">The 2026 standard is not transformation. It is restoration. My goal is that people ask if you have been on vacation, not what you had done. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">DM GLOW to start</t>
@@ -576,7 +599,8 @@
     <t xml:space="preserve">Myth vs Truth: The Frozen Face | The classic fear, debunked.</t>
   </si>
   <si>
-    <t xml:space="preserve">MYTH: Botox freezes your face. TRUTH: correct dosing softens movement while you keep every expression that makes you, you.</t>
+    <t xml:space="preserve">MYTH: Botox freezes your face. TRUTH: correct dosing softens movement while you keep every expression that makes you, you.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Share with a friend</t>
@@ -591,7 +615,8 @@
     <t xml:space="preserve">Client Words: Natural Results | Testimonial card.</t>
   </si>
   <si>
-    <t xml:space="preserve">Nobody could tell. They just kept saying I looked happy and rested. That is the whole goal. 💛 (Shared with permission.)</t>
+    <t xml:space="preserve">Nobody could tell. They just kept saying I looked happy and rested. That is the whole goal. 💛 (Shared with permission.)
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Your turn. Link in bio</t>
@@ -606,7 +631,8 @@
     <t xml:space="preserve">Botox or Filler? You Might Be Asking for the Wrong One | Lines or volume? They are not the same problem.</t>
   </si>
   <si>
-    <t xml:space="preserve">Half the DMs I get ask for the wrong treatment. Here is the simple way to know whether your concern is about movement or volume, and what that means for your plan.</t>
+    <t xml:space="preserve">Half the DMs I get ask for the wrong treatment. Here is the simple way to know whether your concern is about movement or volume, and what that means for your plan.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">DM CONSULT and I will help</t>
@@ -621,7 +647,8 @@
     <t xml:space="preserve">Lines vs Volume | Which one is your concern?</t>
   </si>
   <si>
-    <t xml:space="preserve">Smile in the mirror. Movement lines need Botox. Lost volume needs filler. The answer decides your plan.</t>
+    <t xml:space="preserve">Smile in the mirror. Movement lines need Botox. Lost volume needs filler. The answer decides your plan.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">DM CONSULT for help</t>
@@ -636,7 +663,8 @@
     <t xml:space="preserve">Ask NP Cleo: Your Questions, Answered Honestly | You asked. I answered. No filter.</t>
   </si>
   <si>
-    <t xml:space="preserve">This month you sent amazing questions. Here are the honest answers, including the one nobody else will give you about cheap Botox. Keep them coming. 👇</t>
+    <t xml:space="preserve">This month you sent amazing questions. Here are the honest answers, including the one nobody else will give you about cheap Botox. Keep them coming. 👇
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Drop your question below</t>
@@ -651,7 +679,8 @@
     <t xml:space="preserve">Your DMs, Answered | The question everyone asks quietly.</t>
   </si>
   <si>
-    <t xml:space="preserve">You asked: will people know I had work done? Honest answer: only if you want them to. Subtle is the standard here.</t>
+    <t xml:space="preserve">You asked: will people know I had work done? Honest answer: only if you want them to. Subtle is the standard here.
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Send your question</t>
@@ -666,7 +695,8 @@
     <t xml:space="preserve">Poll: What Should NP Cleo Cover Next? | Audience chooses next month's content.</t>
   </si>
   <si>
-    <t xml:space="preserve">October is filler month. What do you want the truth about first: lips, cheeks, or under eyes? Vote. 👇</t>
+    <t xml:space="preserve">October is filler month. What do you want the truth about first: lips, cheeks, or under eyes? Vote. 👇
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Vote in comments</t>
@@ -681,7 +711,8 @@
     <t xml:space="preserve">How Long Does Botox Really Last? | The honest timeline, month by month.</t>
   </si>
   <si>
-    <t xml:space="preserve">Anyone promising six months is overpromising. Here is the real timeline, what makes it fade faster, and how to make results last longer.</t>
+    <t xml:space="preserve">Anyone promising six months is overpromising. Here is the real timeline, what makes it fade faster, and how to make results last longer.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Save this timeline</t>
@@ -696,7 +727,8 @@
     <t xml:space="preserve">The 3-Month Botox Timeline | Week by week, what to expect.</t>
   </si>
   <si>
-    <t xml:space="preserve">Day 3 it starts. Week 2 it settles. Month 3 it softens. Save this so you know exactly what is normal.</t>
+    <t xml:space="preserve">Day 3 it starts. Week 2 it settles. Month 3 it softens. Save this so you know exactly what is normal.
+#botox #botoxeducation #botoxmyths #preventativebotox #antiwrinkleinjections #nurseinjector #medspa #naturalbotox #botoxbeforeandafter #aestheticnurse</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: timeline infographic card</t>
@@ -711,7 +743,8 @@
     <t xml:space="preserve">Why We Sometimes Say No | A provider who says yes to everyone is a red flag.</t>
   </si>
   <si>
-    <t xml:space="preserve">I have turned people away, and they thanked me later. Here is why honest candidacy matters and what it says about any provider who never says no.</t>
+    <t xml:space="preserve">I have turned people away, and they thanked me later. Here is why honest candidacy matters and what it says about any provider who never says no.
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Book an honest consult</t>
@@ -723,7 +756,8 @@
     <t xml:space="preserve">What I Tell Every First-Timer | The pep talk before every first appointment.</t>
   </si>
   <si>
-    <t xml:space="preserve">You do not need to know the treatment names. You just need to show up honest about your goals. I handle the rest. 💛</t>
+    <t xml:space="preserve">You do not need to know the treatment names. You just need to show up honest about your goals. I handle the rest. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Book your first visit</t>
@@ -738,7 +772,8 @@
     <t xml:space="preserve">Quote: No Is Protection | Brand quote card.</t>
   </si>
   <si>
-    <t xml:space="preserve">An honest provider will sometimes tell you no. That is protection, not rejection. ✨</t>
+    <t xml:space="preserve">An honest provider will sometimes tell you no. That is protection, not rejection. ✨
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Share this</t>
@@ -750,7 +785,8 @@
     <t xml:space="preserve">Filler Won't Make You Look Fake. Bad Technique Does. | The fear is real. The cause is not what you think.</t>
   </si>
   <si>
-    <t xml:space="preserve">Every overdone face you have seen came from heavy hands, not from filler itself. Great work is invisible. You have seen it a hundred times without knowing. ✨</t>
+    <t xml:space="preserve">Every overdone face you have seen came from heavy hands, not from filler itself. Great work is invisible. You have seen it a hundred times without knowing. ✨
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">DM FILLER for a consult</t>
@@ -765,7 +801,8 @@
     <t xml:space="preserve">Service Spotlight: Dermal Filler | Volume where you lost it. Nowhere else.</t>
   </si>
   <si>
-    <t xml:space="preserve">Filler is not about changing your face. It is about restoring what time quietly took. October is filler month. 👀</t>
+    <t xml:space="preserve">Filler is not about changing your face. It is about restoring what time quietly took. October is filler month. 👀
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">DM FILLER to start</t>
@@ -780,7 +817,8 @@
     <t xml:space="preserve">Lip Filler: Natural vs Overdone | The difference is the injector.</t>
   </si>
   <si>
-    <t xml:space="preserve">Soft, balanced, still you. Here is what separates natural lip results from the duck lips everyone fears, and the questions to ask before anyone touches your lips.</t>
+    <t xml:space="preserve">Soft, balanced, still you. Here is what separates natural lip results from the duck lips everyone fears, and the questions to ask before anyone touches your lips.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Save before you book anywhere</t>
@@ -795,7 +833,8 @@
     <t xml:space="preserve">Inside the Filler Appointment | Planned to the last drop.</t>
   </si>
   <si>
-    <t xml:space="preserve">Cannulas, numbing, and a plan drawn before we start. This is what careful looks like.</t>
+    <t xml:space="preserve">Cannulas, numbing, and a plan drawn before we start. This is what careful looks like.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Follow for filler month</t>
@@ -810,7 +849,8 @@
     <t xml:space="preserve">Quote: Subtle Is the New Dramatic | Brand quote card.</t>
   </si>
   <si>
-    <t xml:space="preserve">Subtle is the new dramatic. The best work whispers. 💛</t>
+    <t xml:space="preserve">Subtle is the new dramatic. The best work whispers. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-10-quote-subtle-is-the-new</t>
@@ -819,7 +859,8 @@
     <t xml:space="preserve">Cheek Filler: The Secret Nobody Talks About | The treatment behind the best natural glow-ups.</t>
   </si>
   <si>
-    <t xml:space="preserve">Everyone asks about lips. But cheek filler is quietly behind some of the most natural transformations you have seen. Here is how facial balancing works.</t>
+    <t xml:space="preserve">Everyone asks about lips. But cheek filler is quietly behind some of the most natural transformations you have seen. Here is how facial balancing works.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">DM CHEEKS to learn more</t>
@@ -831,7 +872,8 @@
     <t xml:space="preserve">Service Spotlight: Cheek Filler | The lift nobody talks about.</t>
   </si>
   <si>
-    <t xml:space="preserve">Lifted, refreshed, never puffy. Cheek filler is quietly behind the most natural glow-ups you have seen.</t>
+    <t xml:space="preserve">Lifted, refreshed, never puffy. Cheek filler is quietly behind the most natural glow-ups you have seen.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: cheek treatment photo + hook</t>
@@ -843,7 +885,8 @@
     <t xml:space="preserve">Is Filler Right for You? An Honest Checklist | Not everyone is a candidate. Here is how to know.</t>
   </si>
   <si>
-    <t xml:space="preserve">An honest provider will sometimes tell you not yet. Run through this checklist before your consult and you will walk in knowing exactly what to ask.</t>
+    <t xml:space="preserve">An honest provider will sometimes tell you not yet. Run through this checklist before your consult and you will walk in knowing exactly what to ask.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-15-is-filler-right-for-you</t>
@@ -852,7 +895,8 @@
     <t xml:space="preserve">Facial Balancing 101 | One plan beats three syringes.</t>
   </si>
   <si>
-    <t xml:space="preserve">One syringe in the right place beats three in the wrong ones. Balance first, volume second. Always.</t>
+    <t xml:space="preserve">One syringe in the right place beats three in the wrong ones. Balance first, volume second. Always.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Book a balancing consult</t>
@@ -867,7 +911,8 @@
     <t xml:space="preserve">FAQ: How Much Filler Do I Need? | The honest answer.</t>
   </si>
   <si>
-    <t xml:space="preserve">Less than Instagram makes you think. Most natural results start with one syringe or less. Here is why.</t>
+    <t xml:space="preserve">Less than Instagram makes you think. Most natural results start with one syringe or less. Here is why.
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">More FAQs? DM me</t>
@@ -879,7 +924,8 @@
     <t xml:space="preserve">Filler Dissolves. Here Is the Real Timeline. | What they do not tell you about longevity.</t>
   </si>
   <si>
-    <t xml:space="preserve">Filler is not forever, and that is a feature, not a flaw. Here is how long each area really lasts and what maintenance actually looks like.</t>
+    <t xml:space="preserve">Filler is not forever, and honestly, that is a good thing. Here is how long each area really lasts and what keeping it up actually looks like.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Book your plan. Link in bio</t>
@@ -894,7 +940,8 @@
     <t xml:space="preserve">The Filler Timeline | What happens as it fades.</t>
   </si>
   <si>
-    <t xml:space="preserve">Filler does not vanish overnight and you will not deflate. It softens slowly, on a schedule you can plan around.</t>
+    <t xml:space="preserve">Filler does not vanish overnight and you will not deflate. It softens slowly, on a schedule you can plan around.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-20-the-filler-timeline</t>
@@ -903,7 +950,8 @@
     <t xml:space="preserve">Lip Filler Aftercare: Your First Week | Swelling is normal. Panic is optional.</t>
   </si>
   <si>
-    <t xml:space="preserve">Day 1 looks different from day 7. Here is the honest day-by-day so you know exactly what is normal and when to reach out. Save this before your appointment.</t>
+    <t xml:space="preserve">Day 1 looks different from day 7. Here is the honest day-by-day so you know exactly what is normal and when to reach out. Save this before your appointment.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-22-lip-filler-aftercare-your-first</t>
@@ -912,7 +960,8 @@
     <t xml:space="preserve">Aftercare Essentials | Save this for after your appointment.</t>
   </si>
   <si>
-    <t xml:space="preserve">Ice, no gym for 24 hours, sleep on your back, and message me with anything. That is it. Save this. ✨</t>
+    <t xml:space="preserve">Ice, no gym for 24 hours, sleep on your back, and message me with anything. That is it. Save this. ✨
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Save + share</t>
@@ -927,7 +976,8 @@
     <t xml:space="preserve">Client Words: The Lip Glow-Up | Testimonial card.</t>
   </si>
   <si>
-    <t xml:space="preserve">I finally got my lips done and nobody said filler. They said I looked prettier and could not say why. (Shared with permission.) 💛</t>
+    <t xml:space="preserve">I finally got my lips done and nobody said filler. They said I looked prettier and could not say why. (Shared with permission.) 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Your turn. DM FILLER</t>
@@ -942,7 +992,8 @@
     <t xml:space="preserve">5 Filler Lies You Still Believe | The sequel you asked for.</t>
   </si>
   <si>
-    <t xml:space="preserve">You loved the Botox edition, so here is the filler truth round. Slide 4 is the one that surprises everyone. Share it with your group chat. ✨</t>
+    <t xml:space="preserve">You loved the Botox edition, so here is the filler truth round. Slide 4 is the one that surprises everyone. Share it with your group chat. ✨
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Design in editorial template. Sequel to Botox lies</t>
@@ -954,7 +1005,8 @@
     <t xml:space="preserve">Myth vs Truth: Filler Edition | The one everyone believes.</t>
   </si>
   <si>
-    <t xml:space="preserve">MYTH: filler stretches your lips forever. TRUTH: treated well, your lips return to baseline as filler softens.</t>
+    <t xml:space="preserve">MYTH: filler stretches your lips forever. TRUTH: treated well, your lips return to baseline as filler softens.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Full carousel on our feed</t>
@@ -966,7 +1018,8 @@
     <t xml:space="preserve">Facial Balancing: Why We Treat Faces, Not Lines | Chasing lines is old school.</t>
   </si>
   <si>
-    <t xml:space="preserve">Great aesthetics looks at the whole face: proportions, balance, harmony. Here is why the best results come from a plan, not a single syringe.</t>
+    <t xml:space="preserve">Great aesthetics looks at the whole face: proportions, balance, harmony. Here is why the best results come from a plan, not a single syringe.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">DM BALANCE for a consult</t>
@@ -978,7 +1031,8 @@
     <t xml:space="preserve">Faces, Not Lines | The philosophy behind natural results.</t>
   </si>
   <si>
-    <t xml:space="preserve">Chasing individual lines is old school. Balance and harmony are why my patients look rested instead of done.</t>
+    <t xml:space="preserve">Chasing individual lines is old school. Balance and harmony are why my patients look rested instead of done.
+#dermalfiller #lipfiller #cheekfiller #naturalfiller #facialbalancing #lipfillernatural #aestheticnurse #medspa #fillerjourney #lipgoals</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: philosophy card + portrait</t>
@@ -990,7 +1044,8 @@
     <t xml:space="preserve">Ask Anything: Filler Edition | Engagement post.</t>
   </si>
   <si>
-    <t xml:space="preserve">Filler month is almost over. Drop every remaining question below and I will answer all of them. No judgment. 👇</t>
+    <t xml:space="preserve">Filler month is almost over. Drop every remaining question below and I will answer all of them. No judgment. 👇
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Comment your question</t>
@@ -1011,7 +1066,8 @@
     <t xml:space="preserve">Rested by the Holidays: Your Treatment Timeline | Party season is closer than you think.</t>
   </si>
   <si>
-    <t xml:space="preserve">Botox needs 2 weeks to settle. Filler needs up to 4. If you want to glow in the December photos, here is exactly when to book each treatment. 🗓️</t>
+    <t xml:space="preserve">Botox needs 2 weeks to settle. Filler needs up to 4. If you want to glow in the December photos, here is exactly when to book each treatment. 🗓️
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">Book now. Link in bio</t>
@@ -1029,7 +1085,8 @@
     <t xml:space="preserve">Holiday Countdown: Book by These Dates | Work backwards from party season.</t>
   </si>
   <si>
-    <t xml:space="preserve">Botox needs 2 weeks. Filler needs 4. If you want to glow in the December photos, these are your deadlines. 🗓️</t>
+    <t xml:space="preserve">Botox needs 2 weeks. Filler needs 4. If you want to glow in the December photos, these are your deadlines. 🗓️
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: countdown-dates card</t>
@@ -1041,7 +1098,8 @@
     <t xml:space="preserve">Party Season Prep: What to Book and When | Your holiday glow, planned backwards.</t>
   </si>
   <si>
-    <t xml:space="preserve">Work back from your event date and nothing is rushed, nothing is swollen, and everything looks like you. Here is the smart booking order.</t>
+    <t xml:space="preserve">Work back from your event date and nothing is rushed, nothing is swollen, and everything looks like you. Here is the smart booking order.
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">DM HOLIDAY to book</t>
@@ -1053,7 +1111,8 @@
     <t xml:space="preserve">The Clinic Is Holiday Ready | Glow-up season is officially open.</t>
   </si>
   <si>
-    <t xml:space="preserve">The calendar is filling and the season is here. Your December self will thank your November self. ✨</t>
+    <t xml:space="preserve">The calendar is filling and the season is here. Your December self will thank your November self. ✨
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">Book your spot</t>
@@ -1068,7 +1127,8 @@
     <t xml:space="preserve">Quote: Book the Appointment | Seasonal self-care push.</t>
   </si>
   <si>
-    <t xml:space="preserve">You cannot pour from an empty cup. Book the appointment. Take the hour. You have earned it. 💛</t>
+    <t xml:space="preserve">You cannot pour from an empty cup. Book the appointment. Take the hour. You have earned it. 💛
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">Link in bio</t>
@@ -1080,7 +1140,8 @@
     <t xml:space="preserve">The Gift of Glow: Gift Certificates Are Here | The present nobody returns.</t>
   </si>
   <si>
-    <t xml:space="preserve">Give the people you love something they actually want. Luxury Beauty gift certificates are available in any amount, wrapped and ready. 🎁</t>
+    <t xml:space="preserve">Give the people you love something they actually want. Luxury Beauty gift certificates are available in any amount, wrapped and ready. 🎁
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">DM GIFT to order</t>
@@ -1095,7 +1156,8 @@
     <t xml:space="preserve">Gift Certificates Are Here | The present nobody returns.</t>
   </si>
   <si>
-    <t xml:space="preserve">In any amount, wrapped and beautiful. Give the people you love something they actually want. 🎁</t>
+    <t xml:space="preserve">In any amount, wrapped and beautiful. Give the people you love something they actually want. 🎁
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: gift certificate photo + hook</t>
@@ -1107,7 +1169,8 @@
     <t xml:space="preserve">3 Months of Honest Answers: The Recap | Real education. Real results. Thank you.</t>
   </si>
   <si>
-    <t xml:space="preserve">Since August we have busted myths, answered your questions, and kept every promise about natural results. Here are the posts you loved most, in case you missed one. 💛</t>
+    <t xml:space="preserve">Since August we have busted myths, answered your questions, and kept every promise about natural results. Here are the posts you loved most, in case you missed one. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Follow for what is next</t>
@@ -1122,7 +1185,8 @@
     <t xml:space="preserve">Thank You: 3 Months of Honest Aesthetics | Gratitude post.</t>
   </si>
   <si>
-    <t xml:space="preserve">Since August you have asked incredible questions and trusted us with the answers. Here is to honest aesthetics. Thank you. 💛</t>
+    <t xml:space="preserve">Since August you have asked incredible questions and trusted us with the answers. Here is to honest aesthetics. Thank you. 💛
+#npinjector #nursepractitioner #medspalife #luxurybeauty #aestheticnurse #skincareexpert #beautyclinic #selfcare #naturalresults #honestbeauty</t>
   </si>
   <si>
     <t xml:space="preserve">Single image: team or Cleo photo + thank you overlay</t>
@@ -1134,7 +1198,8 @@
     <t xml:space="preserve">Tag Someone Who Deserves a Glow-Up Gift | Engagement + promo close.</t>
   </si>
   <si>
-    <t xml:space="preserve">Know someone who never treats themselves? Tag them below. We will take care of the rest. 🎁</t>
+    <t xml:space="preserve">Know someone who never treats themselves? Tag them below. We will take care of the rest. 🎁
+#holidayglow #treatyourself #giftcertificate #bookyourappointment #medspaspecial #glowupseason #selfcaregift #luxuryselfcare #holidayready #giftideas</t>
   </si>
   <si>
     <t xml:space="preserve">Tag a friend</t>
@@ -2172,7 +2237,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="9" t="n">
         <v>46251</v>
       </c>
@@ -2222,7 +2287,7 @@
       <c r="S2" s="10"/>
       <c r="T2" s="10"/>
     </row>
-    <row r="3" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="11" t="n">
         <v>46252</v>
       </c>
@@ -2272,7 +2337,7 @@
       <c r="S3" s="12"/>
       <c r="T3" s="12"/>
     </row>
-    <row r="4" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="n">
         <v>46254</v>
       </c>
@@ -2322,7 +2387,7 @@
       <c r="S4" s="10"/>
       <c r="T4" s="10"/>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="11" t="n">
         <v>46255</v>
       </c>
@@ -2372,7 +2437,7 @@
       <c r="S5" s="12"/>
       <c r="T5" s="12"/>
     </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="11" t="n">
         <v>46256</v>
       </c>
@@ -2422,7 +2487,7 @@
       <c r="S6" s="12"/>
       <c r="T6" s="12"/>
     </row>
-    <row r="7" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="n">
         <v>46258</v>
       </c>
@@ -2472,7 +2537,7 @@
       <c r="S7" s="10"/>
       <c r="T7" s="10"/>
     </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="n">
         <v>46259</v>
       </c>
@@ -2522,7 +2587,7 @@
       <c r="S8" s="12"/>
       <c r="T8" s="12"/>
     </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="n">
         <v>46261</v>
       </c>
@@ -2572,7 +2637,7 @@
       <c r="S9" s="10"/>
       <c r="T9" s="10"/>
     </row>
-    <row r="10" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="n">
         <v>46262</v>
       </c>
@@ -2622,7 +2687,7 @@
       <c r="S10" s="12"/>
       <c r="T10" s="12"/>
     </row>
-    <row r="11" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="n">
         <v>46263</v>
       </c>
@@ -2672,7 +2737,7 @@
       <c r="S11" s="12"/>
       <c r="T11" s="12"/>
     </row>
-    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="n">
         <v>46265</v>
       </c>
@@ -2722,7 +2787,7 @@
       <c r="S12" s="10"/>
       <c r="T12" s="10"/>
     </row>
-    <row r="13" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="n">
         <v>46266</v>
       </c>
@@ -2772,7 +2837,7 @@
       <c r="S13" s="12"/>
       <c r="T13" s="12"/>
     </row>
-    <row r="14" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="n">
         <v>46268</v>
       </c>
@@ -2822,7 +2887,7 @@
       <c r="S14" s="10"/>
       <c r="T14" s="10"/>
     </row>
-    <row r="15" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="11" t="n">
         <v>46269</v>
       </c>
@@ -2872,7 +2937,7 @@
       <c r="S15" s="12"/>
       <c r="T15" s="12"/>
     </row>
-    <row r="16" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="n">
         <v>46270</v>
       </c>
@@ -2922,7 +2987,7 @@
       <c r="S16" s="12"/>
       <c r="T16" s="12"/>
     </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="9" t="n">
         <v>46272</v>
       </c>
@@ -2972,7 +3037,7 @@
       <c r="S17" s="10"/>
       <c r="T17" s="10"/>
     </row>
-    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="n">
         <v>46273</v>
       </c>
@@ -3022,7 +3087,7 @@
       <c r="S18" s="12"/>
       <c r="T18" s="12"/>
     </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="9" t="n">
         <v>46275</v>
       </c>
@@ -3072,7 +3137,7 @@
       <c r="S19" s="10"/>
       <c r="T19" s="10"/>
     </row>
-    <row r="20" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="n">
         <v>46276</v>
       </c>
@@ -3122,7 +3187,7 @@
       <c r="S20" s="12"/>
       <c r="T20" s="12"/>
     </row>
-    <row r="21" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="n">
         <v>46277</v>
       </c>
@@ -3172,7 +3237,7 @@
       <c r="S21" s="12"/>
       <c r="T21" s="12"/>
     </row>
-    <row r="22" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="9" t="n">
         <v>46279</v>
       </c>
@@ -3222,7 +3287,7 @@
       <c r="S22" s="10"/>
       <c r="T22" s="10"/>
     </row>
-    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="n">
         <v>46280</v>
       </c>
@@ -3272,7 +3337,7 @@
       <c r="S23" s="12"/>
       <c r="T23" s="12"/>
     </row>
-    <row r="24" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="9" t="n">
         <v>46282</v>
       </c>
@@ -3322,7 +3387,7 @@
       <c r="S24" s="10"/>
       <c r="T24" s="10"/>
     </row>
-    <row r="25" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="n">
         <v>46283</v>
       </c>
@@ -3372,7 +3437,7 @@
       <c r="S25" s="12"/>
       <c r="T25" s="12"/>
     </row>
-    <row r="26" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="n">
         <v>46284</v>
       </c>
@@ -3422,7 +3487,7 @@
       <c r="S26" s="12"/>
       <c r="T26" s="12"/>
     </row>
-    <row r="27" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="9" t="n">
         <v>46286</v>
       </c>
@@ -3472,7 +3537,7 @@
       <c r="S27" s="10"/>
       <c r="T27" s="10"/>
     </row>
-    <row r="28" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="11" t="n">
         <v>46287</v>
       </c>
@@ -3522,7 +3587,7 @@
       <c r="S28" s="12"/>
       <c r="T28" s="12"/>
     </row>
-    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="9" t="n">
         <v>46289</v>
       </c>
@@ -3572,7 +3637,7 @@
       <c r="S29" s="10"/>
       <c r="T29" s="10"/>
     </row>
-    <row r="30" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="11" t="n">
         <v>46290</v>
       </c>
@@ -3622,7 +3687,7 @@
       <c r="S30" s="12"/>
       <c r="T30" s="12"/>
     </row>
-    <row r="31" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="11" t="n">
         <v>46291</v>
       </c>
@@ -3672,7 +3737,7 @@
       <c r="S31" s="12"/>
       <c r="T31" s="12"/>
     </row>
-    <row r="32" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="9" t="n">
         <v>46293</v>
       </c>
@@ -3722,7 +3787,7 @@
       <c r="S32" s="10"/>
       <c r="T32" s="10"/>
     </row>
-    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="11" t="n">
         <v>46294</v>
       </c>
@@ -3772,7 +3837,7 @@
       <c r="S33" s="12"/>
       <c r="T33" s="12"/>
     </row>
-    <row r="34" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="9" t="n">
         <v>46296</v>
       </c>
@@ -3822,7 +3887,7 @@
       <c r="S34" s="10"/>
       <c r="T34" s="10"/>
     </row>
-    <row r="35" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="11" t="n">
         <v>46297</v>
       </c>
@@ -3872,7 +3937,7 @@
       <c r="S35" s="12"/>
       <c r="T35" s="12"/>
     </row>
-    <row r="36" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="11" t="n">
         <v>46298</v>
       </c>
@@ -3922,7 +3987,7 @@
       <c r="S36" s="12"/>
       <c r="T36" s="12"/>
     </row>
-    <row r="37" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="9" t="n">
         <v>46300</v>
       </c>
@@ -3972,7 +4037,7 @@
       <c r="S37" s="10"/>
       <c r="T37" s="10"/>
     </row>
-    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="11" t="n">
         <v>46301</v>
       </c>
@@ -4022,7 +4087,7 @@
       <c r="S38" s="12"/>
       <c r="T38" s="12"/>
     </row>
-    <row r="39" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="9" t="n">
         <v>46303</v>
       </c>
@@ -4072,7 +4137,7 @@
       <c r="S39" s="10"/>
       <c r="T39" s="10"/>
     </row>
-    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="11" t="n">
         <v>46304</v>
       </c>
@@ -4122,7 +4187,7 @@
       <c r="S40" s="12"/>
       <c r="T40" s="12"/>
     </row>
-    <row r="41" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="11" t="n">
         <v>46305</v>
       </c>
@@ -4172,7 +4237,7 @@
       <c r="S41" s="12"/>
       <c r="T41" s="12"/>
     </row>
-    <row r="42" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="42" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="9" t="n">
         <v>46307</v>
       </c>
@@ -4222,7 +4287,7 @@
       <c r="S42" s="10"/>
       <c r="T42" s="10"/>
     </row>
-    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="43" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="11" t="n">
         <v>46308</v>
       </c>
@@ -4272,7 +4337,7 @@
       <c r="S43" s="12"/>
       <c r="T43" s="12"/>
     </row>
-    <row r="44" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="44" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="9" t="n">
         <v>46310</v>
       </c>
@@ -4322,7 +4387,7 @@
       <c r="S44" s="10"/>
       <c r="T44" s="10"/>
     </row>
-    <row r="45" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="11" t="n">
         <v>46311</v>
       </c>
@@ -4372,7 +4437,7 @@
       <c r="S45" s="12"/>
       <c r="T45" s="12"/>
     </row>
-    <row r="46" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="11" t="n">
         <v>46312</v>
       </c>
@@ -4422,7 +4487,7 @@
       <c r="S46" s="12"/>
       <c r="T46" s="12"/>
     </row>
-    <row r="47" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="47" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="9" t="n">
         <v>46314</v>
       </c>
@@ -4472,7 +4537,7 @@
       <c r="S47" s="10"/>
       <c r="T47" s="10"/>
     </row>
-    <row r="48" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="48" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="11" t="n">
         <v>46315</v>
       </c>
@@ -4522,7 +4587,7 @@
       <c r="S48" s="12"/>
       <c r="T48" s="12"/>
     </row>
-    <row r="49" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="9" t="n">
         <v>46317</v>
       </c>
@@ -4572,7 +4637,7 @@
       <c r="S49" s="10"/>
       <c r="T49" s="10"/>
     </row>
-    <row r="50" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="50" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="11" t="n">
         <v>46318</v>
       </c>
@@ -4622,7 +4687,7 @@
       <c r="S50" s="12"/>
       <c r="T50" s="12"/>
     </row>
-    <row r="51" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="51" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="11" t="n">
         <v>46319</v>
       </c>
@@ -4672,7 +4737,7 @@
       <c r="S51" s="12"/>
       <c r="T51" s="12"/>
     </row>
-    <row r="52" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="52" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="9" t="n">
         <v>46321</v>
       </c>
@@ -4722,7 +4787,7 @@
       <c r="S52" s="10"/>
       <c r="T52" s="10"/>
     </row>
-    <row r="53" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="53" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="n">
         <v>46322</v>
       </c>
@@ -4772,7 +4837,7 @@
       <c r="S53" s="12"/>
       <c r="T53" s="12"/>
     </row>
-    <row r="54" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="54" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="9" t="n">
         <v>46324</v>
       </c>
@@ -4822,7 +4887,7 @@
       <c r="S54" s="10"/>
       <c r="T54" s="10"/>
     </row>
-    <row r="55" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="55" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="11" t="n">
         <v>46325</v>
       </c>
@@ -4872,7 +4937,7 @@
       <c r="S55" s="12"/>
       <c r="T55" s="12"/>
     </row>
-    <row r="56" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="n">
         <v>46326</v>
       </c>
@@ -4922,7 +4987,7 @@
       <c r="S56" s="12"/>
       <c r="T56" s="12"/>
     </row>
-    <row r="57" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="57" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="9" t="n">
         <v>46328</v>
       </c>
@@ -4972,7 +5037,7 @@
       <c r="S57" s="10"/>
       <c r="T57" s="10"/>
     </row>
-    <row r="58" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="58" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="11" t="n">
         <v>46329</v>
       </c>
@@ -5022,7 +5087,7 @@
       <c r="S58" s="12"/>
       <c r="T58" s="12"/>
     </row>
-    <row r="59" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="59" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="9" t="n">
         <v>46331</v>
       </c>
@@ -5072,7 +5137,7 @@
       <c r="S59" s="10"/>
       <c r="T59" s="10"/>
     </row>
-    <row r="60" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="60" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="11" t="n">
         <v>46332</v>
       </c>
@@ -5122,7 +5187,7 @@
       <c r="S60" s="12"/>
       <c r="T60" s="12"/>
     </row>
-    <row r="61" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="61" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="n">
         <v>46333</v>
       </c>
@@ -5172,7 +5237,7 @@
       <c r="S61" s="12"/>
       <c r="T61" s="12"/>
     </row>
-    <row r="62" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="62" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="9" t="n">
         <v>46335</v>
       </c>
@@ -5222,7 +5287,7 @@
       <c r="S62" s="10"/>
       <c r="T62" s="10"/>
     </row>
-    <row r="63" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="63" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="11" t="n">
         <v>46336</v>
       </c>
@@ -5272,7 +5337,7 @@
       <c r="S63" s="12"/>
       <c r="T63" s="12"/>
     </row>
-    <row r="64" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="64" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="9" t="n">
         <v>46338</v>
       </c>
@@ -5322,7 +5387,7 @@
       <c r="S64" s="10"/>
       <c r="T64" s="10"/>
     </row>
-    <row r="65" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="65" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="11" t="n">
         <v>46339</v>
       </c>
@@ -5372,7 +5437,7 @@
       <c r="S65" s="12"/>
       <c r="T65" s="12"/>
     </row>
-    <row r="66" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="66" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="11" t="n">
         <v>46340</v>
       </c>

</xml_diff>

<commit_message>
Add jpg copies of all post images and point the sheet at them
Every rendered png in content now has a jpg copy beside it, quality 90. The
set is 23.0MB as png and 6.7MB as jpg, which uploads faster and is the format
Instagram and Google Business Profile prefer anyway. The pngs remain the
render output; the jpgs are what the sheet links to.

Image Link, Preview and GBP Image Link now target the jpg copies, and the
labels say so.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011Bm6abWXhkxKNNCWhPuGt7
</commit_message>
<xml_diff>
--- a/strategy/ig-content-strategy.xlsx
+++ b/strategy/ig-content-strategy.xlsx
@@ -1211,11 +1211,11 @@
       </c>
       <c r="Q2" s="33" t="inlineStr">
         <is>
-          <t>View 8 slides</t>
+          <t>View 8 slides (jpg)</t>
         </is>
       </c>
       <c r="R2" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-17-5-botox-lies-you-still/images/slide-1.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-17-5-botox-lies-you-still/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S2" s="28" t="inlineStr">
@@ -1237,7 +1237,7 @@
       </c>
       <c r="AB2" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -1317,11 +1317,11 @@
       </c>
       <c r="Q3" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R3" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-18-service-spotlight-botox/images/post.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-18-service-spotlight-botox/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S3" s="30" t="inlineStr">
@@ -1343,7 +1343,7 @@
       </c>
       <c r="AB3" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -1429,11 +1429,11 @@
       </c>
       <c r="Q4" s="33" t="inlineStr">
         <is>
-          <t>View 7 slides</t>
+          <t>View 7 slides (jpg)</t>
         </is>
       </c>
       <c r="R4" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-20-5-red-flags-at-a/images/slide-1.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-20-5-red-flags-at-a/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S4" s="28" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="AB4" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -1545,11 +1545,11 @@
       </c>
       <c r="Q5" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R5" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-21-behind-the-scenes-the-prep/images/post.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-21-behind-the-scenes-the-prep/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S5" s="30" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="AB5" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -1665,11 +1665,11 @@
       </c>
       <c r="Q6" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R6" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-22-great-work-is-invisible/images/before-after-result.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-22-great-work-is-invisible/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S6" s="30" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="AB6" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -1782,11 +1782,11 @@
       </c>
       <c r="Q7" s="33" t="inlineStr">
         <is>
-          <t>View 8 slides</t>
+          <t>View 8 slides (jpg)</t>
         </is>
       </c>
       <c r="R7" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-24-your-first-visit-step-by/images/slide-1.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-24-your-first-visit-step-by/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S7" s="28" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="AB7" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -1901,11 +1901,11 @@
       </c>
       <c r="Q8" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R8" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-25-why-i-do-not-post/images/post.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-25-why-i-do-not-post/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S8" s="30" t="inlineStr">
@@ -1931,7 +1931,7 @@
       </c>
       <c r="AB8" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -2018,11 +2018,11 @@
       </c>
       <c r="Q9" s="33" t="inlineStr">
         <is>
-          <t>View 5 slides</t>
+          <t>View 5 slides (jpg)</t>
         </is>
       </c>
       <c r="R9" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-27-meet-np-cleo-the-face/images/slide-1.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-27-meet-np-cleo-the-face/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S9" s="28" t="inlineStr">
@@ -2048,7 +2048,7 @@
       </c>
       <c r="AB9" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -2133,11 +2133,11 @@
       </c>
       <c r="Q10" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R10" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-28-welcome-to-the-treatment-room/images/post.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-28-welcome-to-the-treatment-room/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S10" s="30" t="inlineStr">
@@ -2163,7 +2163,7 @@
       </c>
       <c r="AB10" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -2247,11 +2247,11 @@
       </c>
       <c r="Q11" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R11" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-29-this-or-that-rested-vs/images/post.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-29-this-or-that-rested-vs/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S11" s="30" t="inlineStr">
@@ -2277,7 +2277,7 @@
       </c>
       <c r="AB11" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -2364,11 +2364,11 @@
       </c>
       <c r="Q12" s="33" t="inlineStr">
         <is>
-          <t>View 7 slides</t>
+          <t>View 7 slides (jpg)</t>
         </is>
       </c>
       <c r="R12" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-31-preventative-botox-when-to-actually/images/slide-1.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-08-31-preventative-botox-when-to-actually/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S12" s="28" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="AB12" s="33" t="inlineStr">
         <is>
-          <t>View GBP image</t>
+          <t>View GBP image (jpg)</t>
         </is>
       </c>
     </row>
@@ -5052,11 +5052,11 @@
       </c>
       <c r="Q39" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R39" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-08-lip-filler-natural-vs-overdone/images/before-after-result.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-08-lip-filler-natural-vs-overdone/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S39" s="28" t="inlineStr">
@@ -5257,11 +5257,11 @@
       </c>
       <c r="Q41" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R41" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-10-subtle-is-the-new-dramatic/images/before-after-result.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-10-subtle-is-the-new-dramatic/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S41" s="30" t="inlineStr">
@@ -5561,11 +5561,11 @@
       </c>
       <c r="Q44" s="33" t="inlineStr">
         <is>
-          <t>View 7 slides</t>
+          <t>View 7 slides (jpg)</t>
         </is>
       </c>
       <c r="R44" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-15-real-lips-real-results/images/slide-1.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-15-real-lips-real-results/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S44" s="28" t="inlineStr">
@@ -6063,11 +6063,11 @@
       </c>
       <c r="Q49" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R49" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-22-lip-filler-aftercare-your-first/images/day-zero-before-after.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-22-lip-filler-aftercare-your-first/images/day-zero-before-after.jpg")</f>
         <v/>
       </c>
       <c r="S49" s="28" t="inlineStr">
@@ -6268,11 +6268,11 @@
       </c>
       <c r="Q51" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R51" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-24-client-words-the-lip-glow/images/before-after-result.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-24-client-words-the-lip-glow/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S51" s="30" t="inlineStr">
@@ -6671,11 +6671,11 @@
       </c>
       <c r="Q55" s="33" t="inlineStr">
         <is>
-          <t>View image</t>
+          <t>View image (jpg)</t>
         </is>
       </c>
       <c r="R55" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-30-one-syringe-balanced-lips/images/before-after-result.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-10-30-one-syringe-balanced-lips/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S55" s="30" t="inlineStr">
@@ -7173,11 +7173,11 @@
       </c>
       <c r="Q60" s="33" t="inlineStr">
         <is>
-          <t>View 7 slides</t>
+          <t>View 7 slides (jpg)</t>
         </is>
       </c>
       <c r="R60" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-11-06-one-result-every-angle/images/slide-1.png")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/convert-images-jpg-5jeayb/content/2026-11-06-one-result-every-angle/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S60" s="30" t="inlineStr">
@@ -7802,98 +7802,127 @@
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P2" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId11"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId12"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId13"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA7" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA8" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA9" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA10" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA12" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P51" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q2" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA2" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB2" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O3" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P3" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q3" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA3" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB3" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O4" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P4" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q4" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA4" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB4" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O5" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P5" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q5" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA5" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB5" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O6" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P6" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q6" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA6" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB6" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O7" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P7" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q7" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA7" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB7" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O8" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P8" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q8" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA8" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB8" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O9" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P9" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q9" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA9" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB9" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O10" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P10" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA10" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB10" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O11" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P11" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O12" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P12" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA12" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB12" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O13" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O14" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O15" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O16" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O17" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O18" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O19" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O20" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O21" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O22" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O23" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O24" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O26" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O28" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O29" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O30" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O31" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O32" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O33" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O34" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O35" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O36" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O37" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O38" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O39" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P39" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q39" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O40" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O41" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P41" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q41" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O42" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O43" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P44" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q44" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P49" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q49" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P51" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q51" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P55" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q55" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="P60" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q60" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId123"/>
   </hyperlinks>
   <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Point the planner links at the default branch
The image and folder links were pinned to this feature branch, which goes
away once the work lands. They now point at claude/med-spa-carousel-ideas-sim9wz,
the branch the repo actually opens on, so the Preview and Image Link columns
keep resolving after the merge.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XrNeahC933uq1i2byuFHGy
</commit_message>
<xml_diff>
--- a/strategy/ig-content-strategy.xlsx
+++ b/strategy/ig-content-strategy.xlsx
@@ -1201,7 +1201,7 @@
       <c r="N2" s="24" t="n"/>
       <c r="O2" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-17-5-botox-lies-you-still</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-17-5-botox-lies-you-still</t>
         </is>
       </c>
       <c r="P2" s="32" t="inlineStr">
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="R2" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-17-5-botox-lies-you-still/images/slide-1.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-17-5-botox-lies-you-still/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S2" s="28" t="inlineStr">
@@ -1232,7 +1232,7 @@
       <c r="Z2" s="24" t="n"/>
       <c r="AA2" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/blob/claude/image-size-format-instagram-855nfc/content/2026-08-17-5-botox-lies-you-still/images/gbp.jpg?raw=1</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/blob/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-17-5-botox-lies-you-still/images/gbp.jpg?raw=1</t>
         </is>
       </c>
       <c r="AB2" s="33" t="inlineStr">
@@ -1307,7 +1307,7 @@
       <c r="N3" s="24" t="n"/>
       <c r="O3" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-18-service-spotlight-botox</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-18-service-spotlight-botox</t>
         </is>
       </c>
       <c r="P3" s="34" t="inlineStr">
@@ -1321,7 +1321,7 @@
         </is>
       </c>
       <c r="R3" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-18-service-spotlight-botox/images/post.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-18-service-spotlight-botox/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S3" s="30" t="inlineStr">
@@ -1338,7 +1338,7 @@
       <c r="Z3" s="24" t="n"/>
       <c r="AA3" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/blob/claude/image-size-format-instagram-855nfc/content/2026-08-18-service-spotlight-botox/images/gbp.jpg?raw=1</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/blob/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-18-service-spotlight-botox/images/gbp.jpg?raw=1</t>
         </is>
       </c>
       <c r="AB3" s="33" t="inlineStr">
@@ -1419,7 +1419,7 @@
       <c r="N4" s="24" t="n"/>
       <c r="O4" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-20-5-red-flags-at-a</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-20-5-red-flags-at-a</t>
         </is>
       </c>
       <c r="P4" s="32" t="inlineStr">
@@ -1433,7 +1433,7 @@
         </is>
       </c>
       <c r="R4" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-20-5-red-flags-at-a/images/slide-1.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-20-5-red-flags-at-a/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S4" s="28" t="inlineStr">
@@ -1535,7 +1535,7 @@
       <c r="N5" s="24" t="n"/>
       <c r="O5" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-21-behind-the-scenes-the-prep</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-21-behind-the-scenes-the-prep</t>
         </is>
       </c>
       <c r="P5" s="34" t="inlineStr">
@@ -1549,7 +1549,7 @@
         </is>
       </c>
       <c r="R5" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-21-behind-the-scenes-the-prep/images/post.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-21-behind-the-scenes-the-prep/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S5" s="30" t="inlineStr">
@@ -1669,7 +1669,7 @@
         </is>
       </c>
       <c r="R6" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-22-great-work-is-invisible/images/before-after-result.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-22-great-work-is-invisible/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S6" s="30" t="inlineStr">
@@ -1772,7 +1772,7 @@
       <c r="N7" s="24" t="n"/>
       <c r="O7" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-24-your-first-visit-step-by</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-24-your-first-visit-step-by</t>
         </is>
       </c>
       <c r="P7" s="32" t="inlineStr">
@@ -1786,7 +1786,7 @@
         </is>
       </c>
       <c r="R7" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-24-your-first-visit-step-by/images/slide-1.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-24-your-first-visit-step-by/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S7" s="28" t="inlineStr">
@@ -1891,7 +1891,7 @@
       <c r="N8" s="24" t="n"/>
       <c r="O8" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-25-why-i-do-not-post</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-25-why-i-do-not-post</t>
         </is>
       </c>
       <c r="P8" s="34" t="inlineStr">
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="R8" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-25-why-i-do-not-post/images/post.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-25-why-i-do-not-post/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S8" s="30" t="inlineStr">
@@ -2008,7 +2008,7 @@
       <c r="N9" s="24" t="n"/>
       <c r="O9" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-27-meet-np-cleo-the-face</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-27-meet-np-cleo-the-face</t>
         </is>
       </c>
       <c r="P9" s="32" t="inlineStr">
@@ -2022,7 +2022,7 @@
         </is>
       </c>
       <c r="R9" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-27-meet-np-cleo-the-face/images/slide-1.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-27-meet-np-cleo-the-face/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S9" s="28" t="inlineStr">
@@ -2123,7 +2123,7 @@
       <c r="N10" s="24" t="n"/>
       <c r="O10" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-28-welcome-to-the-treatment-room</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-28-welcome-to-the-treatment-room</t>
         </is>
       </c>
       <c r="P10" s="34" t="inlineStr">
@@ -2137,7 +2137,7 @@
         </is>
       </c>
       <c r="R10" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-28-welcome-to-the-treatment-room/images/post.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-28-welcome-to-the-treatment-room/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S10" s="30" t="inlineStr">
@@ -2237,7 +2237,7 @@
       <c r="N11" s="24" t="n"/>
       <c r="O11" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-29-this-or-that-rested-vs</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-29-this-or-that-rested-vs</t>
         </is>
       </c>
       <c r="P11" s="34" t="inlineStr">
@@ -2251,7 +2251,7 @@
         </is>
       </c>
       <c r="R11" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-29-this-or-that-rested-vs/images/post.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-29-this-or-that-rested-vs/images/post.jpg")</f>
         <v/>
       </c>
       <c r="S11" s="30" t="inlineStr">
@@ -2354,7 +2354,7 @@
       <c r="N12" s="24" t="n"/>
       <c r="O12" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-08-31-preventative-botox-when-to-actually</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-31-preventative-botox-when-to-actually</t>
         </is>
       </c>
       <c r="P12" s="32" t="inlineStr">
@@ -2368,7 +2368,7 @@
         </is>
       </c>
       <c r="R12" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-08-31-preventative-botox-when-to-actually/images/slide-1.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-08-31-preventative-botox-when-to-actually/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S12" s="28" t="inlineStr">
@@ -2464,7 +2464,7 @@
       <c r="N13" s="24" t="n"/>
       <c r="O13" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-01-service-spotlight-preventative-botox</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-01-service-spotlight-preventative-botox</t>
         </is>
       </c>
       <c r="P13" s="34" t="inlineStr">
@@ -2563,7 +2563,7 @@
       <c r="N14" s="24" t="n"/>
       <c r="O14" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-03-what-20-units-actually-looks</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-03-what-20-units-actually-looks</t>
         </is>
       </c>
       <c r="P14" s="32" t="inlineStr">
@@ -2662,7 +2662,7 @@
       <c r="N15" s="24" t="n"/>
       <c r="O15" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-04-meet-your-injector</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-04-meet-your-injector</t>
         </is>
       </c>
       <c r="P15" s="34" t="inlineStr">
@@ -2761,7 +2761,7 @@
       <c r="N16" s="24" t="n"/>
       <c r="O16" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-05-quote-prevention-beats-erasing</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-05-quote-prevention-beats-erasing</t>
         </is>
       </c>
       <c r="P16" s="34" t="inlineStr">
@@ -2860,7 +2860,7 @@
       <c r="N17" s="24" t="n"/>
       <c r="O17" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-07-botox-vs-dysport-the-real</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-07-botox-vs-dysport-the-real</t>
         </is>
       </c>
       <c r="P17" s="32" t="inlineStr">
@@ -2959,7 +2959,7 @@
       <c r="N18" s="24" t="n"/>
       <c r="O18" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-08-botox-vs-dysport-at-a</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-08-botox-vs-dysport-at-a</t>
         </is>
       </c>
       <c r="P18" s="34" t="inlineStr">
@@ -3058,7 +3058,7 @@
       <c r="N19" s="24" t="n"/>
       <c r="O19" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-10-botox-aftercare-the-first-48</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-10-botox-aftercare-the-first-48</t>
         </is>
       </c>
       <c r="P19" s="32" t="inlineStr">
@@ -3157,7 +3157,7 @@
       <c r="N20" s="24" t="n"/>
       <c r="O20" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-11-the-face-map</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-11-the-face-map</t>
         </is>
       </c>
       <c r="P20" s="34" t="inlineStr">
@@ -3256,7 +3256,7 @@
       <c r="N21" s="24" t="n"/>
       <c r="O21" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-12-faq-does-botox-hurt</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-12-faq-does-botox-hurt</t>
         </is>
       </c>
       <c r="P21" s="34" t="inlineStr">
@@ -3355,7 +3355,7 @@
       <c r="N22" s="24" t="n"/>
       <c r="O22" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-14-5-things-botox-can-t</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-14-5-things-botox-can-t</t>
         </is>
       </c>
       <c r="P22" s="32" t="inlineStr">
@@ -3454,7 +3454,7 @@
       <c r="N23" s="24" t="n"/>
       <c r="O23" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-15-what-botox-can-t-fix</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-15-what-botox-can-t-fix</t>
         </is>
       </c>
       <c r="P23" s="34" t="inlineStr">
@@ -3553,7 +3553,7 @@
       <c r="N24" s="24" t="n"/>
       <c r="O24" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-17-still-you-just-refreshed</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-17-still-you-just-refreshed</t>
         </is>
       </c>
       <c r="P24" s="32" t="inlineStr">
@@ -3652,7 +3652,7 @@
       <c r="N25" s="24" t="n"/>
       <c r="O25" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-18-myth-vs-truth-the-frozen</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-18-myth-vs-truth-the-frozen</t>
         </is>
       </c>
       <c r="P25" s="34" t="inlineStr">
@@ -3751,7 +3751,7 @@
       <c r="N26" s="24" t="n"/>
       <c r="O26" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-19-client-words-natural-results</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-19-client-words-natural-results</t>
         </is>
       </c>
       <c r="P26" s="34" t="inlineStr">
@@ -3850,7 +3850,7 @@
       <c r="N27" s="24" t="n"/>
       <c r="O27" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-21-botox-or-filler-you-might</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-21-botox-or-filler-you-might</t>
         </is>
       </c>
       <c r="P27" s="32" t="inlineStr">
@@ -3949,7 +3949,7 @@
       <c r="N28" s="24" t="n"/>
       <c r="O28" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-22-lines-vs-volume</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-22-lines-vs-volume</t>
         </is>
       </c>
       <c r="P28" s="34" t="inlineStr">
@@ -4048,7 +4048,7 @@
       <c r="N29" s="24" t="n"/>
       <c r="O29" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-24-ask-np-cleo-your-questions</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-24-ask-np-cleo-your-questions</t>
         </is>
       </c>
       <c r="P29" s="32" t="inlineStr">
@@ -4147,7 +4147,7 @@
       <c r="N30" s="24" t="n"/>
       <c r="O30" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-25-your-dms-answered</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-25-your-dms-answered</t>
         </is>
       </c>
       <c r="P30" s="34" t="inlineStr">
@@ -4246,7 +4246,7 @@
       <c r="N31" s="24" t="n"/>
       <c r="O31" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-26-poll-what-should-np-cleo</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-26-poll-what-should-np-cleo</t>
         </is>
       </c>
       <c r="P31" s="34" t="inlineStr">
@@ -4345,7 +4345,7 @@
       <c r="N32" s="24" t="n"/>
       <c r="O32" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-28-how-long-does-botox-really</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-28-how-long-does-botox-really</t>
         </is>
       </c>
       <c r="P32" s="32" t="inlineStr">
@@ -4444,7 +4444,7 @@
       <c r="N33" s="24" t="n"/>
       <c r="O33" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-09-29-the-3-month-botox-timeline</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-09-29-the-3-month-botox-timeline</t>
         </is>
       </c>
       <c r="P33" s="34" t="inlineStr">
@@ -4543,7 +4543,7 @@
       <c r="N34" s="24" t="n"/>
       <c r="O34" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-01-why-we-sometimes-say-no</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-01-why-we-sometimes-say-no</t>
         </is>
       </c>
       <c r="P34" s="32" t="inlineStr">
@@ -4642,7 +4642,7 @@
       <c r="N35" s="24" t="n"/>
       <c r="O35" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-02-what-i-tell-every-first</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-02-what-i-tell-every-first</t>
         </is>
       </c>
       <c r="P35" s="34" t="inlineStr">
@@ -4741,7 +4741,7 @@
       <c r="N36" s="24" t="n"/>
       <c r="O36" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-03-quote-no-is-protection</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-03-quote-no-is-protection</t>
         </is>
       </c>
       <c r="P36" s="34" t="inlineStr">
@@ -4840,7 +4840,7 @@
       <c r="N37" s="24" t="n"/>
       <c r="O37" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-05-filler-won-t-make-you</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-05-filler-won-t-make-you</t>
         </is>
       </c>
       <c r="P37" s="32" t="inlineStr">
@@ -4939,7 +4939,7 @@
       <c r="N38" s="24" t="n"/>
       <c r="O38" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-06-service-spotlight-dermal-filler</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-06-service-spotlight-dermal-filler</t>
         </is>
       </c>
       <c r="P38" s="34" t="inlineStr">
@@ -5056,7 +5056,7 @@
         </is>
       </c>
       <c r="R39" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-10-08-lip-filler-natural-vs-overdone/images/before-after-result.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-08-lip-filler-natural-vs-overdone/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S39" s="28" t="inlineStr">
@@ -5144,7 +5144,7 @@
       <c r="N40" s="24" t="n"/>
       <c r="O40" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-09-inside-the-filler-appointment</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-09-inside-the-filler-appointment</t>
         </is>
       </c>
       <c r="P40" s="34" t="inlineStr">
@@ -5261,7 +5261,7 @@
         </is>
       </c>
       <c r="R41" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-10-10-subtle-is-the-new-dramatic/images/before-after-result.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-10-subtle-is-the-new-dramatic/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S41" s="30" t="inlineStr">
@@ -5349,7 +5349,7 @@
       <c r="N42" s="24" t="n"/>
       <c r="O42" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-12-cheek-filler-the-secret-nobody</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-12-cheek-filler-the-secret-nobody</t>
         </is>
       </c>
       <c r="P42" s="32" t="inlineStr">
@@ -5448,7 +5448,7 @@
       <c r="N43" s="24" t="n"/>
       <c r="O43" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-13-service-spotlight-cheek-filler</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-13-service-spotlight-cheek-filler</t>
         </is>
       </c>
       <c r="P43" s="34" t="inlineStr">
@@ -5565,7 +5565,7 @@
         </is>
       </c>
       <c r="R44" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-10-15-real-lips-real-results/images/slide-1.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-15-real-lips-real-results/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S44" s="28" t="inlineStr">
@@ -5653,7 +5653,7 @@
       <c r="N45" s="24" t="n"/>
       <c r="O45" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-16-facial-balancing-101</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-16-facial-balancing-101</t>
         </is>
       </c>
       <c r="P45" s="34" t="inlineStr">
@@ -5752,7 +5752,7 @@
       <c r="N46" s="24" t="n"/>
       <c r="O46" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-17-faq-how-much-filler-do</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-17-faq-how-much-filler-do</t>
         </is>
       </c>
       <c r="P46" s="34" t="inlineStr">
@@ -5851,7 +5851,7 @@
       <c r="N47" s="24" t="n"/>
       <c r="O47" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-19-filler-dissolves-here-is-the</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-19-filler-dissolves-here-is-the</t>
         </is>
       </c>
       <c r="P47" s="32" t="inlineStr">
@@ -5950,7 +5950,7 @@
       <c r="N48" s="24" t="n"/>
       <c r="O48" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-20-the-filler-timeline</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-20-the-filler-timeline</t>
         </is>
       </c>
       <c r="P48" s="34" t="inlineStr">
@@ -6067,7 +6067,7 @@
         </is>
       </c>
       <c r="R49" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-10-22-lip-filler-aftercare-your-first/images/day-zero-before-after.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-22-lip-filler-aftercare-your-first/images/day-zero-before-after.jpg")</f>
         <v/>
       </c>
       <c r="S49" s="28" t="inlineStr">
@@ -6155,7 +6155,7 @@
       <c r="N50" s="24" t="n"/>
       <c r="O50" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-23-aftercare-essentials</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-23-aftercare-essentials</t>
         </is>
       </c>
       <c r="P50" s="34" t="inlineStr">
@@ -6272,7 +6272,7 @@
         </is>
       </c>
       <c r="R51" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-10-24-client-words-the-lip-glow/images/before-after-result.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-24-client-words-the-lip-glow/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S51" s="30" t="inlineStr">
@@ -6360,7 +6360,7 @@
       <c r="N52" s="24" t="n"/>
       <c r="O52" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-26-5-filler-lies-you-still</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-26-5-filler-lies-you-still</t>
         </is>
       </c>
       <c r="P52" s="32" t="inlineStr">
@@ -6459,7 +6459,7 @@
       <c r="N53" s="24" t="n"/>
       <c r="O53" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-27-myth-vs-truth-filler-edition</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-27-myth-vs-truth-filler-edition</t>
         </is>
       </c>
       <c r="P53" s="34" t="inlineStr">
@@ -6558,7 +6558,7 @@
       <c r="N54" s="24" t="n"/>
       <c r="O54" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-29-facial-balancing-why-we-treat</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-29-facial-balancing-why-we-treat</t>
         </is>
       </c>
       <c r="P54" s="32" t="inlineStr">
@@ -6675,7 +6675,7 @@
         </is>
       </c>
       <c r="R55" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-10-30-one-syringe-balanced-lips/images/before-after-result.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-30-one-syringe-balanced-lips/images/before-after-result.jpg")</f>
         <v/>
       </c>
       <c r="S55" s="30" t="inlineStr">
@@ -6763,7 +6763,7 @@
       <c r="N56" s="24" t="n"/>
       <c r="O56" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-10-31-ask-anything-filler-edition</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-10-31-ask-anything-filler-edition</t>
         </is>
       </c>
       <c r="P56" s="34" t="inlineStr">
@@ -6862,7 +6862,7 @@
       <c r="N57" s="24" t="n"/>
       <c r="O57" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-02-rested-by-the-holidays-your</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-02-rested-by-the-holidays-your</t>
         </is>
       </c>
       <c r="P57" s="32" t="inlineStr">
@@ -6961,7 +6961,7 @@
       <c r="N58" s="24" t="n"/>
       <c r="O58" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-03-holiday-countdown-book-by-these</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-03-holiday-countdown-book-by-these</t>
         </is>
       </c>
       <c r="P58" s="34" t="inlineStr">
@@ -7060,7 +7060,7 @@
       <c r="N59" s="24" t="n"/>
       <c r="O59" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-05-party-season-prep-what-to</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-05-party-season-prep-what-to</t>
         </is>
       </c>
       <c r="P59" s="32" t="inlineStr">
@@ -7177,7 +7177,7 @@
         </is>
       </c>
       <c r="R60" s="24">
-        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/image-size-format-instagram-855nfc/content/2026-11-06-one-result-every-angle/images/slide-1.jpg")</f>
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-06-one-result-every-angle/images/slide-1.jpg")</f>
         <v/>
       </c>
       <c r="S60" s="30" t="inlineStr">
@@ -7265,7 +7265,7 @@
       <c r="N61" s="24" t="n"/>
       <c r="O61" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-07-quote-book-the-appointment</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-07-quote-book-the-appointment</t>
         </is>
       </c>
       <c r="P61" s="34" t="inlineStr">
@@ -7364,7 +7364,7 @@
       <c r="N62" s="24" t="n"/>
       <c r="O62" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-09-the-gift-of-glow-gift</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-09-the-gift-of-glow-gift</t>
         </is>
       </c>
       <c r="P62" s="32" t="inlineStr">
@@ -7463,7 +7463,7 @@
       <c r="N63" s="24" t="n"/>
       <c r="O63" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-10-gift-certificates-are-here</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-10-gift-certificates-are-here</t>
         </is>
       </c>
       <c r="P63" s="34" t="inlineStr">
@@ -7562,7 +7562,7 @@
       <c r="N64" s="24" t="n"/>
       <c r="O64" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-12-3-months-of-honest-answers</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-12-3-months-of-honest-answers</t>
         </is>
       </c>
       <c r="P64" s="32" t="inlineStr">
@@ -7661,7 +7661,7 @@
       <c r="N65" s="24" t="n"/>
       <c r="O65" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-13-thank-you-3-months-of</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-13-thank-you-3-months-of</t>
         </is>
       </c>
       <c r="P65" s="34" t="inlineStr">
@@ -7760,7 +7760,7 @@
       <c r="N66" s="24" t="n"/>
       <c r="O66" s="24" t="inlineStr">
         <is>
-          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/image-size-format-instagram-855nfc/content/2026-11-14-tag-someone-who-deserves-a</t>
+          <t>https://github.com/RepoKing23/InstagramCarousel/tree/claude/med-spa-carousel-ideas-sim9wz/content/2026-11-14-tag-someone-who-deserves-a</t>
         </is>
       </c>
       <c r="P66" s="34" t="inlineStr">

</xml_diff>

<commit_message>
Extend the GBP calendar through October, and print the copy
October follows the Instagram grid into filler month: 31 more daily cards,
Oct 1 to Oct 31, taking the run to 74 days. Twenty three of them carry that
day's Instagram message rewritten for someone who found the clinic on Maps,
and the eight Wednesdays and Sundays are evergreen, filler safety, candidacy,
bruising, pricing, how to book and where the studio is.

Every October day gets both lengths of copy, the same as the existing set,
and the whole month uses all 23 photos with no repeat closer than twelve
days. Layout check passes on all 74 cards.

Also: the Sep 28 long copy carried the same paragraph twice, now removed.

New, design/build-blog-copy.py writes strategy/gbp-blog-copy.md, the entire
run of copy as one readable document so it can be read or handed on without
opening the workbook.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017DLHmdZ9wPpFHL1RPBs8zc
</commit_message>
<xml_diff>
--- a/strategy/ig-content-strategy.xlsx
+++ b/strategy/ig-content-strategy.xlsx
@@ -8157,7 +8157,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q44"/>
+  <dimension ref="A1:Q75"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="14" min="1" max="1"/>
@@ -11455,12 +11455,11 @@
         <is>
           <t>Three to four months for most people, and here are the honest reasons it varies.
 Metabolism plays a part, and people who train hard often find it wears off sooner. Dose matters, since a light preventative dose fades before a fuller corrective one. Muscle strength matters, because a strong frown works through product faster than a light one. And history matters, as people who have treated consistently for years often stretch further between appointments.
-What is not true is that it stops working. If yours seems to be fading faster than it used to, the usual answer is that the dose is no longer right rather than any resistance to the product.
 What is not true is that it stops working. If your Botox seems to be fading faster than it used to, the usual answer is that the dose is no longer right rather than any resistance to the product. Month by month timeline on Instagram.</t>
         </is>
       </c>
       <c r="H42" s="45" t="n">
-        <v>885</v>
+        <v>693</v>
       </c>
       <c r="I42" s="45" t="inlineStr">
         <is>
@@ -11660,6 +11659,2455 @@
         </is>
       </c>
       <c r="Q44" s="42" t="inlineStr"/>
+    </row>
+    <row r="45" ht="132" customHeight="1" s="14">
+      <c r="A45" s="51" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B45" s="45" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C45" s="45" t="inlineStr">
+        <is>
+          <t>IG: Why We Sometimes Say No</t>
+        </is>
+      </c>
+      <c r="D45" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E45" s="46" t="inlineStr">
+        <is>
+          <t>I have turned people away from filler and had them thank me later. Some faces do not need it, and some do not need it yet. Candidacy is part of the assessment, not a step on the way to a sale. The full post is on Instagram.</t>
+        </is>
+      </c>
+      <c r="F45" s="45" t="n">
+        <v>223</v>
+      </c>
+      <c r="G45" s="46" t="inlineStr">
+        <is>
+          <t>I have turned people away from filler, and they thanked me later.
+Some faces do not need it. Some do not need it yet. And some are asking filler to fix something filler does not fix, usually skin quality or a heavy lower face that needs a different plan entirely. Saying yes to all three is easy. It is also how people end up with a result that never sat right and money spent twice.
+Candidacy is part of the assessment at our Oakville studio, not a step on the way to a sale. If I do not think you will be happy in six months, I will tell you at the consult and it costs you nothing.
+A provider who has never said no to anyone is telling you something. The full post is on Instagram.</t>
+        </is>
+      </c>
+      <c r="H45" s="45" t="n">
+        <v>687</v>
+      </c>
+      <c r="I45" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J45" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K45" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-01-why-i-say-no.jpg</t>
+        </is>
+      </c>
+      <c r="L45" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M45" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N45" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-01-why-i-say-no.jpg")</f>
+        <v/>
+      </c>
+      <c r="O45" s="47" t="inlineStr">
+        <is>
+          <t>Look Studio / Unsplash</t>
+        </is>
+      </c>
+      <c r="P45" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q45" s="46" t="inlineStr"/>
+    </row>
+    <row r="46" ht="132" customHeight="1" s="14">
+      <c r="A46" s="51" t="n">
+        <v>46297</v>
+      </c>
+      <c r="B46" s="45" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C46" s="45" t="inlineStr">
+        <is>
+          <t>IG: What I Tell Every First-Timer</t>
+        </is>
+      </c>
+      <c r="D46" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E46" s="46" t="inlineStr">
+        <is>
+          <t>The same four things I tell every first time filler client. Start smaller than you think, judge it at two weeks, swelling is not your result, and you can always add. Nobody regrets going conservative first. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F46" s="45" t="n">
+        <v>220</v>
+      </c>
+      <c r="G46" s="46" t="inlineStr">
+        <is>
+          <t>Four things I tell every first time filler client in Oakville, before anything is opened.
+Start smaller than you think. A partial syringe is a real option and a good one. Judge it at two weeks, not at day two, because what you see in the first 48 hours is swelling and not your result. Nothing about the first appointment has to be the final answer, since we can add at the review.
+And the last one, which matters most: tell me what you actually want to look like, not which treatment you think you want. The plan is my job. The goal is yours.
+Nobody has ever regretted going conservative on their first syringe. Book a consult, or read the full post on Instagram.</t>
+        </is>
+      </c>
+      <c r="H46" s="45" t="n">
+        <v>667</v>
+      </c>
+      <c r="I46" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J46" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K46" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-02-every-first-timer.jpg</t>
+        </is>
+      </c>
+      <c r="L46" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M46" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N46" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-02-every-first-timer.jpg")</f>
+        <v/>
+      </c>
+      <c r="O46" s="47" t="inlineStr">
+        <is>
+          <t>karelys Ruiz / Unsplash</t>
+        </is>
+      </c>
+      <c r="P46" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q46" s="46" t="inlineStr"/>
+    </row>
+    <row r="47" ht="132" customHeight="1" s="14">
+      <c r="A47" s="51" t="n">
+        <v>46298</v>
+      </c>
+      <c r="B47" s="45" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C47" s="45" t="inlineStr">
+        <is>
+          <t>IG: Quote: No Is Protection</t>
+        </is>
+      </c>
+      <c r="D47" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E47" s="46" t="inlineStr">
+        <is>
+          <t>No is protection. It is the most underrated part of good injecting and the hardest thing to hear from someone you were ready to pay. A provider willing to lose the booking is the one worth booking. More on Instagram.</t>
+        </is>
+      </c>
+      <c r="F47" s="45" t="n">
+        <v>216</v>
+      </c>
+      <c r="G47" s="46" t="inlineStr">
+        <is>
+          <t>No is protection. It is the most underrated part of good injecting.
+It is also the hardest thing to hear from a provider you were already prepared to pay. Nobody arrives at a consult hoping to be told to wait, or to be told the thing they read about is not the thing their face needs. But the alternative is worse, and it is the reason a certain kind of result is recognisable across a room.
+A nurse practitioner willing to lose the booking is the one worth booking. That is the whole of it.
+If you have been told yes to everything you have ever asked for, that is not a compliment to your face. It is information about the person holding the syringe. More on Instagram, or come and ask in Oakville.</t>
+        </is>
+      </c>
+      <c r="H47" s="45" t="n">
+        <v>702</v>
+      </c>
+      <c r="I47" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J47" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K47" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-03-no-is-protection.jpg</t>
+        </is>
+      </c>
+      <c r="L47" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M47" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N47" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-03-no-is-protection.jpg")</f>
+        <v/>
+      </c>
+      <c r="O47" s="47" t="inlineStr">
+        <is>
+          <t>engin akyurt / Unsplash</t>
+        </is>
+      </c>
+      <c r="P47" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q47" s="46" t="inlineStr"/>
+    </row>
+    <row r="48" ht="132" customHeight="1" s="14">
+      <c r="A48" s="50" t="n">
+        <v>46299</v>
+      </c>
+      <c r="B48" s="41" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C48" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D48" s="41" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E48" s="42" t="inlineStr">
+        <is>
+          <t>The honest answer on filler safety. The fillers I use are hyaluronic acid, which the body already makes and which can be dissolved if a result is not right. Safety comes from the injector, the assessment and the anatomy. More on Instagram.</t>
+        </is>
+      </c>
+      <c r="F48" s="41" t="n">
+        <v>239</v>
+      </c>
+      <c r="G48" s="42" t="inlineStr">
+        <is>
+          <t>The honest answer on filler safety, without the sales gloss.
+The fillers used at the Oakville studio are hyaluronic acid, a substance the body already makes. That matters for one specific reason: it can be dissolved. If a result is not right, or settles unevenly, there is a way back. That is not true of every product on the market, which is exactly why I use these ones.
+The real safety question is not the product, it is the person holding the syringe and whether they know the anatomy underneath. Filler goes near vessels. Placement is the whole job.
+Injections here are done by a nurse practitioner and never delegated. Bring your questions to the consult, including the uncomfortable ones.</t>
+        </is>
+      </c>
+      <c r="H48" s="41" t="n">
+        <v>698</v>
+      </c>
+      <c r="I48" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J48" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K48" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-04-is-filler-safe.jpg</t>
+        </is>
+      </c>
+      <c r="L48" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M48" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N48" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-04-is-filler-safe.jpg")</f>
+        <v/>
+      </c>
+      <c r="O48" s="43" t="inlineStr">
+        <is>
+          <t>Look Studio / Unsplash</t>
+        </is>
+      </c>
+      <c r="P48" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q48" s="42" t="inlineStr"/>
+    </row>
+    <row r="49" ht="132" customHeight="1" s="14">
+      <c r="A49" s="51" t="n">
+        <v>46300</v>
+      </c>
+      <c r="B49" s="45" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C49" s="45" t="inlineStr">
+        <is>
+          <t>IG: Filler Won't Make You Look Fake</t>
+        </is>
+      </c>
+      <c r="D49" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E49" s="46" t="inlineStr">
+        <is>
+          <t>Filler is not what makes a face look fake. Volume in the wrong place, too much at once, and treating one feature while ignoring the rest are what make a face look done. The technique is the variable, not the product. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F49" s="45" t="n">
+        <v>230</v>
+      </c>
+      <c r="G49" s="46" t="inlineStr">
+        <is>
+          <t>Filler does not make a face look fake. Technique does.
+The three things that actually cause it: too much product at one sitting, product placed in the wrong plane or the wrong compartment, and chasing one feature while the rest of the face is ignored. Lips built on a face that has lost midface support will always read as lips first, no matter how carefully they are shaped.
+This is why the assessment looks at the whole face even when you came in asking about one part of it. Balance is the point, and volume is only ever a means to it.
+The results people admire and cannot identify are filler too. You just never got told. See the full carousel on Instagram, or book an assessment in Oakville.</t>
+        </is>
+      </c>
+      <c r="H49" s="45" t="n">
+        <v>699</v>
+      </c>
+      <c r="I49" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J49" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K49" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-05-fake-is-not-the-filler.jpg</t>
+        </is>
+      </c>
+      <c r="L49" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M49" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N49" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-05-fake-is-not-the-filler.jpg")</f>
+        <v/>
+      </c>
+      <c r="O49" s="47" t="inlineStr">
+        <is>
+          <t>JEaLiFe Pictures / Unsplash</t>
+        </is>
+      </c>
+      <c r="P49" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q49" s="46" t="inlineStr"/>
+    </row>
+    <row r="50" ht="132" customHeight="1" s="14">
+      <c r="A50" s="51" t="n">
+        <v>46301</v>
+      </c>
+      <c r="B50" s="45" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C50" s="45" t="inlineStr">
+        <is>
+          <t>IG: Service Spotlight: Dermal Filler</t>
+        </is>
+      </c>
+      <c r="D50" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E50" s="46" t="inlineStr">
+        <is>
+          <t>Dermal filler, plainly. It replaces volume the face has lost or shapes what was always a little short, which is a different job from Botox. Lips, cheeks, chin and jawline, injected by a nurse practitioner in Oakville. See the spotlight on Instagram.</t>
+        </is>
+      </c>
+      <c r="F50" s="45" t="n">
+        <v>249</v>
+      </c>
+      <c r="G50" s="46" t="inlineStr">
+        <is>
+          <t>Dermal filler, explained plainly, because it gets confused with Botox constantly.
+Botox relaxes muscle, so it softens lines that movement creates. Filler adds structure, so it replaces volume the face has lost or shapes what was always a little short. Different problems, different tools, and plenty of faces need neither yet.
+At the Oakville studio I treat lips, cheeks, chin and jawline with hyaluronic acid filler, injected by a nurse practitioner and never delegated to anyone else.
+Most first appointments are one syringe or less. Results are visible immediately, settle over about two weeks, and last somewhere between six and eighteen months depending on the area and how your body handles it. See the spotlight on Instagram.</t>
+        </is>
+      </c>
+      <c r="H50" s="45" t="n">
+        <v>735</v>
+      </c>
+      <c r="I50" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J50" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K50" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-06-spotlight-dermal-filler.jpg</t>
+        </is>
+      </c>
+      <c r="L50" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M50" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N50" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-06-spotlight-dermal-filler.jpg")</f>
+        <v/>
+      </c>
+      <c r="O50" s="47" t="inlineStr">
+        <is>
+          <t>Elist Nguyen / Unsplash</t>
+        </is>
+      </c>
+      <c r="P50" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q50" s="46" t="inlineStr"/>
+    </row>
+    <row r="51" ht="132" customHeight="1" s="14">
+      <c r="A51" s="50" t="n">
+        <v>46302</v>
+      </c>
+      <c r="B51" s="41" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C51" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D51" s="41" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E51" s="42" t="inlineStr">
+        <is>
+          <t>What a filler consult includes at our Oakville studio. A full face assessment, your history and medications, an honest read on candidacy, a plan with an area and an amount, and a price before anything is opened. You can leave without booking.</t>
+        </is>
+      </c>
+      <c r="F51" s="41" t="n">
+        <v>242</v>
+      </c>
+      <c r="G51" s="42" t="inlineStr">
+        <is>
+          <t>What a filler consult includes, before anything is opened.
+We start with what is bothering you, in your words. Then a full face assessment, because the answer is often not where the complaint is. Then your health history and medications, since blood thinners and a few other things change the plan and the bruising risk.
+You leave with an area, an amount, a price and a realistic idea of what it will and will not do. If the honest answer is not yet, or not this, you get that instead, and it costs you nothing.
+No product is opened until you have agreed to the plan and the price. Nobody is talked into anything in this room. The studio is on Preserve Dr in Oakville, with free parking at the door.</t>
+        </is>
+      </c>
+      <c r="H51" s="41" t="n">
+        <v>702</v>
+      </c>
+      <c r="I51" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J51" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K51" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-07-before-the-syringe.jpg</t>
+        </is>
+      </c>
+      <c r="L51" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M51" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N51" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-07-before-the-syringe.jpg")</f>
+        <v/>
+      </c>
+      <c r="O51" s="43" t="inlineStr">
+        <is>
+          <t>Rosa Rafael / Unsplash</t>
+        </is>
+      </c>
+      <c r="P51" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q51" s="42" t="inlineStr"/>
+    </row>
+    <row r="52" ht="132" customHeight="1" s="14">
+      <c r="A52" s="51" t="n">
+        <v>46303</v>
+      </c>
+      <c r="B52" s="45" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C52" s="45" t="inlineStr">
+        <is>
+          <t>IG: Lip Filler: Natural vs Overdone</t>
+        </is>
+      </c>
+      <c r="D52" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E52" s="46" t="inlineStr">
+        <is>
+          <t>Natural versus overdone lips, side by side. The difference is ratio and shape, not the brand of filler. Respect the border, keep the lower fuller than the upper, and stop before it is obvious. Shared with client consent on Instagram.</t>
+        </is>
+      </c>
+      <c r="F52" s="45" t="n">
+        <v>233</v>
+      </c>
+      <c r="G52" s="46" t="inlineStr">
+        <is>
+          <t>Natural or overdone. The difference is ratio and shape, not the product.
+A lip that reads as natural keeps its border, keeps the lower lip fuller than the upper, and keeps the height of the upper lip in proportion to the space above it. A lip that reads as done usually broke one of those three, most often by filling past the border or by adding volume that the lip could not carry.
+Amount matters less than people assume. I have seen a full syringe look untouched and half of one look obvious, and the variable both times was placement.
+The lip filler work worth showing is the kind nobody identifies as work. Real examples, shared with client consent, are on Instagram. Assessments in Oakville.</t>
+        </is>
+      </c>
+      <c r="H52" s="45" t="n">
+        <v>700</v>
+      </c>
+      <c r="I52" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J52" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K52" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-08-natural-or-overdone.jpg</t>
+        </is>
+      </c>
+      <c r="L52" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M52" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N52" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-08-natural-or-overdone.jpg")</f>
+        <v/>
+      </c>
+      <c r="O52" s="47" t="inlineStr">
+        <is>
+          <t>Fleur Kaan / Unsplash</t>
+        </is>
+      </c>
+      <c r="P52" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q52" s="46" t="inlineStr"/>
+    </row>
+    <row r="53" ht="132" customHeight="1" s="14">
+      <c r="A53" s="51" t="n">
+        <v>46304</v>
+      </c>
+      <c r="B53" s="45" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C53" s="45" t="inlineStr">
+        <is>
+          <t>IG: Inside the Filler Appointment</t>
+        </is>
+      </c>
+      <c r="D53" s="45" t="inlineStr">
+        <is>
+          <t>Personality &amp; BTS</t>
+        </is>
+      </c>
+      <c r="E53" s="46" t="inlineStr">
+        <is>
+          <t>What a filler appointment actually looks like. Photos, numbing cream for around twenty minutes, mapping while it works, then injecting in small increments with a mirror check as we go. About forty five minutes door to door. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F53" s="45" t="n">
+        <v>237</v>
+      </c>
+      <c r="G53" s="46" t="inlineStr">
+        <is>
+          <t>What a filler appointment actually looks like, start to finish.
+Photos first, because memory is unreliable and you will want the comparison. Numbing cream for about twenty minutes, and I map the face while it works. Then the injecting, done in small increments with a mirror in your hand at the checkpoints, not one long uninterrupted run.
+Most of the appointment is not the needle. Around forty five minutes door to door for a single area, and you leave with ice, aftercare in writing and my number.
+The part people are surprised by is how much talking there is in the middle of it. Adjusting as we go is not indecision, it is how a symmetrical result happens. Come and see the room on Instagram, or book in Oakville.</t>
+        </is>
+      </c>
+      <c r="H53" s="45" t="n">
+        <v>721</v>
+      </c>
+      <c r="I53" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J53" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K53" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-09-inside-the-appointment.jpg</t>
+        </is>
+      </c>
+      <c r="L53" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M53" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N53" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-09-inside-the-appointment.jpg")</f>
+        <v/>
+      </c>
+      <c r="O53" s="47" t="inlineStr">
+        <is>
+          <t>Anuruddha Lokuhapuarachchi / Unsplash</t>
+        </is>
+      </c>
+      <c r="P53" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q53" s="46" t="inlineStr"/>
+    </row>
+    <row r="54" ht="132" customHeight="1" s="14">
+      <c r="A54" s="51" t="n">
+        <v>46305</v>
+      </c>
+      <c r="B54" s="45" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C54" s="45" t="inlineStr">
+        <is>
+          <t>IG: Subtle Is the New Dramatic</t>
+        </is>
+      </c>
+      <c r="D54" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E54" s="46" t="inlineStr">
+        <is>
+          <t>Subtle is not a compromise, it is the goal. If the first thing anyone notices about your face is the filler, something in the plan was wrong. A real result, shared with client consent, is on Instagram.</t>
+        </is>
+      </c>
+      <c r="F54" s="45" t="n">
+        <v>201</v>
+      </c>
+      <c r="G54" s="46" t="inlineStr">
+        <is>
+          <t>Subtle is not a compromise. It is the goal.
+The dramatic result is easy. Anyone can add volume until a change is undeniable. The difficult version is the one where your face looks rested and balanced and nobody can name what changed, which takes restraint, an honest read of proportion, and a willingness to stop early.
+If the first thing people notice about you is your filler, the plan was wrong before the needle came out.
+This is the standard everything at the Oakville studio is held to. Half a syringe placed properly beats a full one placed to be seen, every single time. A real result, shared with the client's consent, is on Instagram. Assessments for lips, cheeks and jawline are booked the same way.</t>
+        </is>
+      </c>
+      <c r="H54" s="45" t="n">
+        <v>713</v>
+      </c>
+      <c r="I54" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J54" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K54" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-10-subtle-is-the-point.jpg</t>
+        </is>
+      </c>
+      <c r="L54" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M54" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N54" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-10-subtle-is-the-point.jpg")</f>
+        <v/>
+      </c>
+      <c r="O54" s="47" t="inlineStr">
+        <is>
+          <t>Fleur Kaan / Unsplash</t>
+        </is>
+      </c>
+      <c r="P54" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q54" s="46" t="inlineStr"/>
+    </row>
+    <row r="55" ht="132" customHeight="1" s="14">
+      <c r="A55" s="50" t="n">
+        <v>46306</v>
+      </c>
+      <c r="B55" s="41" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C55" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D55" s="41" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E55" s="42" t="inlineStr">
+        <is>
+          <t>We are at 3060 Preserve Dr in Oakville, a private studio rather than a clinic floor, with free parking at the door. Clients come from Burlington, Milton and Mississauga for Botox and filler. Appointment only, evenings available.</t>
+        </is>
+      </c>
+      <c r="F55" s="41" t="n">
+        <v>228</v>
+      </c>
+      <c r="G55" s="42" t="inlineStr">
+        <is>
+          <t>A private studio in Oakville, not a clinic floor and not a shopping centre counter.
+We are at 3060 Preserve Dr, with free parking directly outside and no lobby to sit in. Appointments are one at a time, which is why the schedule is by booking only and why nobody is ever rushed through.
+Clients drive in from Burlington, Milton and Mississauga, and a good number from north Oakville who did not know there was anything closer than the QEW.
+Botox, dermal filler, lip filler and cheek filler, all injected by a nurse practitioner. Evening appointments are available for people coming after work, which is most of them. Send a message on Instagram to book, or ask for directions and I will send them.</t>
+        </is>
+      </c>
+      <c r="H55" s="41" t="n">
+        <v>700</v>
+      </c>
+      <c r="I55" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J55" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K55" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-11-find-the-studio.jpg</t>
+        </is>
+      </c>
+      <c r="L55" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M55" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N55" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-11-find-the-studio.jpg")</f>
+        <v/>
+      </c>
+      <c r="O55" s="43" t="inlineStr">
+        <is>
+          <t>Wco Global / Unsplash</t>
+        </is>
+      </c>
+      <c r="P55" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q55" s="42" t="inlineStr"/>
+    </row>
+    <row r="56" ht="132" customHeight="1" s="14">
+      <c r="A56" s="51" t="n">
+        <v>46307</v>
+      </c>
+      <c r="B56" s="45" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C56" s="45" t="inlineStr">
+        <is>
+          <t>IG: Cheek Filler: The Secret Nobody Talks About</t>
+        </is>
+      </c>
+      <c r="D56" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E56" s="46" t="inlineStr">
+        <is>
+          <t>The cheek is the most underrated area on the face. Support the midface and the lower face softens, because half of what looks heavy at the jaw is really volume that dropped from above. Most people ask for the wrong area first. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F56" s="45" t="n">
+        <v>240</v>
+      </c>
+      <c r="G56" s="46" t="inlineStr">
+        <is>
+          <t>Cheeks hold the face up. That is the part nobody talks about.
+When the midface loses volume, the tissue below it has less to sit on, so it settles. That is why the lines at the mouth deepen, why the lower face starts reading heavy, and why treating either one directly often does very little. The problem is above where you are looking.
+Restore midface support and the lower face lifts with it. No filler in the lower face at all, and it still softens.
+This is the most common redirection I make at consults in Oakville. Someone comes in asking about the lines around the mouth and leaves with a plan for cheeks, and it is a smaller amount of product than they expected. The full explanation is on Instagram.</t>
+        </is>
+      </c>
+      <c r="H56" s="45" t="n">
+        <v>711</v>
+      </c>
+      <c r="I56" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J56" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K56" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-12-cheeks-hold-the-face.jpg</t>
+        </is>
+      </c>
+      <c r="L56" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M56" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N56" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-12-cheeks-hold-the-face.jpg")</f>
+        <v/>
+      </c>
+      <c r="O56" s="47" t="inlineStr">
+        <is>
+          <t>Elist Nguyen / Unsplash</t>
+        </is>
+      </c>
+      <c r="P56" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q56" s="46" t="inlineStr"/>
+    </row>
+    <row r="57" ht="132" customHeight="1" s="14">
+      <c r="A57" s="51" t="n">
+        <v>46308</v>
+      </c>
+      <c r="B57" s="45" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C57" s="45" t="inlineStr">
+        <is>
+          <t>IG: Service Spotlight: Cheek Filler</t>
+        </is>
+      </c>
+      <c r="D57" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E57" s="46" t="inlineStr">
+        <is>
+          <t>Cheek filler in Oakville, explained. Placed deep for structure rather than fullness, it restores the support the midface has lost. Usually one syringe, results visible immediately, settled by two weeks, lasting twelve to eighteen months. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F57" s="45" t="n">
+        <v>251</v>
+      </c>
+      <c r="G57" s="46" t="inlineStr">
+        <is>
+          <t>Cheek filler is structure, not volume. That distinction is the entire treatment.
+Placed deep, on bone, it restores the support the midface lost rather than sitting shallow and making a face look fuller. Done well it reads as looking rested and slightly lifted. Done shallow or done too much, it reads as cheeks, which is the version everyone has seen and nobody wants.
+Most cheek appointments at the Oakville studio are one syringe, sometimes split across two visits so we can assess in between.
+Results are visible the same day, settle over about two weeks, and typically last twelve to eighteen months, longer than lips because the area moves less. Injected by a nurse practitioner. See the spotlight on Instagram.</t>
+        </is>
+      </c>
+      <c r="H57" s="45" t="n">
+        <v>719</v>
+      </c>
+      <c r="I57" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J57" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K57" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-13-spotlight-cheek-filler.jpg</t>
+        </is>
+      </c>
+      <c r="L57" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M57" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N57" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-13-spotlight-cheek-filler.jpg")</f>
+        <v/>
+      </c>
+      <c r="O57" s="47" t="inlineStr">
+        <is>
+          <t>Zac Taheriyan / Unsplash</t>
+        </is>
+      </c>
+      <c r="P57" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q57" s="46" t="inlineStr"/>
+    </row>
+    <row r="58" ht="132" customHeight="1" s="14">
+      <c r="A58" s="50" t="n">
+        <v>46309</v>
+      </c>
+      <c r="B58" s="41" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C58" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D58" s="41" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E58" s="42" t="inlineStr">
+        <is>
+          <t>Filler is not right for everyone, and not right for everyone today. Pregnancy and breastfeeding, an active skin infection at the site, certain medications and an event too close to the date are all reasons I will ask you to wait. Ask at the consult.</t>
+        </is>
+      </c>
+      <c r="F58" s="41" t="n">
+        <v>249</v>
+      </c>
+      <c r="G58" s="42" t="inlineStr">
+        <is>
+          <t>Filler is not right for everyone, and not right for everyone today.
+The clear ones: pregnancy and breastfeeding, an active skin infection or breakout at the injection site, and a recent dental procedure, which we sit out for two weeks in either direction. Some medications change the plan rather than cancel it, blood thinners in particular, so bring your full list to the consult.
+Timing is the one people fight me on. A wedding in ten days is not the week to start, because bruising and swelling need room.
+The other reason to wait is simply that your face does not need it yet, which is a real answer and one I give often at the Oakville studio. Ask me directly and you will get a direct answer.</t>
+        </is>
+      </c>
+      <c r="H58" s="41" t="n">
+        <v>701</v>
+      </c>
+      <c r="I58" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J58" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K58" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-14-not-everyone-is-a-candidate.jpg</t>
+        </is>
+      </c>
+      <c r="L58" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M58" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N58" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-14-not-everyone-is-a-candidate.jpg")</f>
+        <v/>
+      </c>
+      <c r="O58" s="43" t="inlineStr">
+        <is>
+          <t>Masum Rahimi / Unsplash</t>
+        </is>
+      </c>
+      <c r="P58" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q58" s="42" t="inlineStr"/>
+    </row>
+    <row r="59" ht="132" customHeight="1" s="14">
+      <c r="A59" s="51" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B59" s="45" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C59" s="45" t="inlineStr">
+        <is>
+          <t>IG: Real Lips. Real Results.</t>
+        </is>
+      </c>
+      <c r="D59" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E59" s="46" t="inlineStr">
+        <is>
+          <t>Real lip filler results from the Oakville studio, shared with written client consent. Same lighting, same angle, no filter, no smoothing. Some are half a syringe. This is what the work actually looks like. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F59" s="45" t="n">
+        <v>219</v>
+      </c>
+      <c r="G59" s="46" t="inlineStr">
+        <is>
+          <t>Real lips, real results, shared with written client consent.
+Every comparison is the same lighting, the same angle and the same distance, with no filter and no smoothing. That is a low bar and it should be standard, but it is not, which is why the change in some of these will look smaller than what you see elsewhere. Smaller is the point.
+A few of these are half a syringe. One is a correction of somebody else's work, and that is labelled, because it is a different job with a different starting point.
+If you want to know what lip filler in Oakville actually looks like on ordinary faces rather than on a screen, this is the honest version. The full set is on Instagram, and consultations are booked from there.</t>
+        </is>
+      </c>
+      <c r="H59" s="45" t="n">
+        <v>718</v>
+      </c>
+      <c r="I59" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J59" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K59" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-15-real-lips-real-results.jpg</t>
+        </is>
+      </c>
+      <c r="L59" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M59" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N59" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-15-real-lips-real-results.jpg")</f>
+        <v/>
+      </c>
+      <c r="O59" s="47" t="inlineStr">
+        <is>
+          <t>Vitaliy Shevchenko / Unsplash</t>
+        </is>
+      </c>
+      <c r="P59" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q59" s="46" t="inlineStr"/>
+    </row>
+    <row r="60" ht="132" customHeight="1" s="14">
+      <c r="A60" s="51" t="n">
+        <v>46311</v>
+      </c>
+      <c r="B60" s="45" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C60" s="45" t="inlineStr">
+        <is>
+          <t>IG: Facial Balancing 101</t>
+        </is>
+      </c>
+      <c r="D60" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E60" s="46" t="inlineStr">
+        <is>
+          <t>Facial balancing, in one post. It treats the relationship between features rather than the one feature that bothers you. A chin that is slightly short changes how the lips read, so treating the lips alone would have chased the wrong thing. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F60" s="45" t="n">
+        <v>253</v>
+      </c>
+      <c r="G60" s="46" t="inlineStr">
+        <is>
+          <t>Facial balancing treats proportion, not the feature you came in about.
+Here is the version that makes it click. A chin that sits slightly short makes the lower lip look like it is projecting further than it is, so someone comes in asking to have their upper lip built to match. Do that and you have made both problems worse. Support the chin and the lips read as balanced without touching them.
+The same logic runs through the midface, the jawline and the temples. Features are read against each other, never on their own.
+This is why a consult in Oakville looks at the whole face even when your question is about one part of it, and why the plan is often a smaller amount of product in a different place. The full explanation is on Instagram.</t>
+        </is>
+      </c>
+      <c r="H60" s="45" t="n">
+        <v>746</v>
+      </c>
+      <c r="I60" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J60" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K60" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-16-facial-balancing-101.jpg</t>
+        </is>
+      </c>
+      <c r="L60" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M60" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N60" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-16-facial-balancing-101.jpg")</f>
+        <v/>
+      </c>
+      <c r="O60" s="47" t="inlineStr">
+        <is>
+          <t>Masum Rahimi / Unsplash</t>
+        </is>
+      </c>
+      <c r="P60" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q60" s="46" t="inlineStr"/>
+    </row>
+    <row r="61" ht="132" customHeight="1" s="14">
+      <c r="A61" s="51" t="n">
+        <v>46312</v>
+      </c>
+      <c r="B61" s="45" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C61" s="45" t="inlineStr">
+        <is>
+          <t>IG: FAQ: How Much Filler Do I Need?</t>
+        </is>
+      </c>
+      <c r="D61" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E61" s="46" t="inlineStr">
+        <is>
+          <t>How much filler do you need? Usually less than you think. One syringe is roughly a fifth of a teaspoon, and for lips that is often a full result or more than one appointment needs. Half syringes are a real option here. Details on Instagram.</t>
+        </is>
+      </c>
+      <c r="F61" s="45" t="n">
+        <v>240</v>
+      </c>
+      <c r="G61" s="46" t="inlineStr">
+        <is>
+          <t>How much filler do I need? Almost always less than you think.
+One syringe is about a millilitre, which is roughly a fifth of a teaspoon. On lips that is frequently a complete result, and for a first appointment half of one is often the better call. Cheeks usually take a full syringe per side over time, though rarely all at once. Chin and jawline sit somewhere in between.
+The number that matters is not how many syringes, it is how much your face can carry before it stops looking like your face.
+At the Oakville studio I would rather you come back in a month and add than sit with too much for the next year. Filler dissolves, but waiting it out is nobody's idea of a good outcome. Ask at the consult, or read the FAQ on Instagram.</t>
+        </is>
+      </c>
+      <c r="H61" s="45" t="n">
+        <v>737</v>
+      </c>
+      <c r="I61" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J61" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K61" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-17-how-much-do-i-need.jpg</t>
+        </is>
+      </c>
+      <c r="L61" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M61" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N61" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-17-how-much-do-i-need.jpg")</f>
+        <v/>
+      </c>
+      <c r="O61" s="47" t="inlineStr">
+        <is>
+          <t>Victor Meza / Unsplash</t>
+        </is>
+      </c>
+      <c r="P61" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q61" s="46" t="inlineStr"/>
+    </row>
+    <row r="62" ht="132" customHeight="1" s="14">
+      <c r="A62" s="50" t="n">
+        <v>46313</v>
+      </c>
+      <c r="B62" s="41" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C62" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D62" s="41" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E62" s="42" t="inlineStr">
+        <is>
+          <t>How to arrive for filler. Eat beforehand, skip alcohol for 24 hours, hold fish oil and ibuprofen if your doctor allows, come with a clean face and leave the evening plans open. Small things, and they change how the next two days go.</t>
+        </is>
+      </c>
+      <c r="F62" s="41" t="n">
+        <v>232</v>
+      </c>
+      <c r="G62" s="42" t="inlineStr">
+        <is>
+          <t>How to arrive for a filler appointment, so the next two days go easier.
+Eat first. People who come in on an empty stomach are the ones who feel lightheaded. Skip alcohol for the 24 hours before, since it thins the blood and bruising follows. If your own doctor is fine with it, hold fish oil, high dose vitamin E and ibuprofen for a few days beforehand, and never stop a prescribed blood thinner without asking them.
+Come with a clean face. Makeup goes off before we start anyway, so save yourself the step.
+And leave the evening open. You will look swollen, possibly uneven, and that is the treatment working rather than the result. Appointments at the Oakville studio run about forty five minutes, including numbing.</t>
+        </is>
+      </c>
+      <c r="H62" s="41" t="n">
+        <v>721</v>
+      </c>
+      <c r="I62" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J62" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K62" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-18-on-the-day-itself.jpg</t>
+        </is>
+      </c>
+      <c r="L62" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M62" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N62" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-18-on-the-day-itself.jpg")</f>
+        <v/>
+      </c>
+      <c r="O62" s="43" t="inlineStr">
+        <is>
+          <t>Christin Hume / Unsplash</t>
+        </is>
+      </c>
+      <c r="P62" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q62" s="42" t="inlineStr"/>
+    </row>
+    <row r="63" ht="132" customHeight="1" s="14">
+      <c r="A63" s="51" t="n">
+        <v>46314</v>
+      </c>
+      <c r="B63" s="45" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C63" s="45" t="inlineStr">
+        <is>
+          <t>IG: Filler Dissolves. Here Is the Real Timeline.</t>
+        </is>
+      </c>
+      <c r="D63" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E63" s="46" t="inlineStr">
+        <is>
+          <t>Filler is not permanent. Lips run six to twelve months, cheeks and jawline twelve to eighteen, because areas that move more break product down faster. And hyaluronic acid can be dissolved deliberately if a result is wrong. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F63" s="45" t="n">
+        <v>236</v>
+      </c>
+      <c r="G63" s="46" t="inlineStr">
+        <is>
+          <t>Filler dissolves. Here is the real timeline, area by area.
+Lips run about six to twelve months, because the mouth never stops moving and movement breaks product down. Cheeks and jawline run twelve to eighteen for the opposite reason. Chin sits near the longer end. Your metabolism moves all of those numbers, and people who train hard usually sit at the short end of every range.
+What does not happen is filler disappearing overnight. It softens gradually, which is why people think it lasted longer than it did.
+And the part that should be said more often: hyaluronic acid filler can be dissolved deliberately, in one appointment, if a result is not right. That is not a hypothetical safety net, it is a treatment I actually perform in Oakville. Full timeline on Instagram.</t>
+        </is>
+      </c>
+      <c r="H63" s="45" t="n">
+        <v>777</v>
+      </c>
+      <c r="I63" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J63" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K63" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-19-it-dissolves.jpg</t>
+        </is>
+      </c>
+      <c r="L63" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M63" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N63" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-19-it-dissolves.jpg")</f>
+        <v/>
+      </c>
+      <c r="O63" s="47" t="inlineStr">
+        <is>
+          <t>Alef Morais / Unsplash</t>
+        </is>
+      </c>
+      <c r="P63" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q63" s="46" t="inlineStr"/>
+    </row>
+    <row r="64" ht="132" customHeight="1" s="14">
+      <c r="A64" s="51" t="n">
+        <v>46315</v>
+      </c>
+      <c r="B64" s="45" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C64" s="45" t="inlineStr">
+        <is>
+          <t>IG: The Filler Timeline</t>
+        </is>
+      </c>
+      <c r="D64" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E64" s="46" t="inlineStr">
+        <is>
+          <t>Day by day after lip filler. Day one is swollen and firm, day two is often the peak, by day three it is settling, bruising clears through week one, and two weeks is your actual result. Judge it then, not before. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F64" s="45" t="n">
+        <v>225</v>
+      </c>
+      <c r="G64" s="46" t="inlineStr">
+        <is>
+          <t>Day one swollen. Day three settling. Two weeks is your result.
+Day one, expect firm and larger than the final shape, sometimes noticeably uneven. Day two is the swelling peak for most people, which is the day everybody messages me. Day three it begins to come down and starts to look like a lip again. Any bruising surfaces and clears through the first week.
+Week two is when the product has fully integrated and the shape is real. That is the only fair point to judge it, and the point at which we review.
+The day two panic is the single most common message I get after lip filler in Oakville, and it is almost never a problem. Save the timeline from Instagram so you have it on your phone when you need it.</t>
+        </is>
+      </c>
+      <c r="H64" s="45" t="n">
+        <v>711</v>
+      </c>
+      <c r="I64" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J64" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K64" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-20-the-filler-timeline.jpg</t>
+        </is>
+      </c>
+      <c r="L64" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M64" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N64" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-20-the-filler-timeline.jpg")</f>
+        <v/>
+      </c>
+      <c r="O64" s="47" t="inlineStr">
+        <is>
+          <t>Zulfugar Karimov / Unsplash</t>
+        </is>
+      </c>
+      <c r="P64" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q64" s="46" t="inlineStr"/>
+    </row>
+    <row r="65" ht="132" customHeight="1" s="14">
+      <c r="A65" s="50" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B65" s="41" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C65" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D65" s="41" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E65" s="42" t="inlineStr">
+        <is>
+          <t>Will filler bruise? Sometimes, and it is not a sign anything went wrong. Lips bruise most because the tissue is vascular. Skip alcohol beforehand, hold blood thinning supplements if your doctor agrees, ice after, and expect it clear within a week.</t>
+        </is>
+      </c>
+      <c r="F65" s="41" t="n">
+        <v>247</v>
+      </c>
+      <c r="G65" s="42" t="inlineStr">
+        <is>
+          <t>Will I bruise? Sometimes, and it does not mean anything went wrong.
+Filler is placed in tissue that has blood vessels running through it, and lips have more of them than anywhere else I treat. A needle can meet one. Careful technique lowers the odds and no technique removes them, which is why I will not promise you a bruise free appointment.
+What helps: no alcohol for 24 hours beforehand, holding fish oil, vitamin E and ibuprofen for a few days if your own doctor agrees, ice afterwards, and arnica if you like it.
+Most bruising is small, most of it is coverable with makeup after 24 hours, and nearly all of it is gone inside a week. Book with a week of room before anything you care about, and you will never have to think about it.</t>
+        </is>
+      </c>
+      <c r="H65" s="41" t="n">
+        <v>741</v>
+      </c>
+      <c r="I65" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J65" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K65" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-21-will-i-bruise.jpg</t>
+        </is>
+      </c>
+      <c r="L65" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M65" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N65" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-21-will-i-bruise.jpg")</f>
+        <v/>
+      </c>
+      <c r="O65" s="43" t="inlineStr">
+        <is>
+          <t>Neda Vidakovic / Unsplash</t>
+        </is>
+      </c>
+      <c r="P65" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q65" s="42" t="inlineStr"/>
+    </row>
+    <row r="66" ht="132" customHeight="1" s="14">
+      <c r="A66" s="51" t="n">
+        <v>46317</v>
+      </c>
+      <c r="B66" s="45" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C66" s="45" t="inlineStr">
+        <is>
+          <t>IG: Lip Filler Aftercare: Your First Week</t>
+        </is>
+      </c>
+      <c r="D66" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E66" s="46" t="inlineStr">
+        <is>
+          <t>Lip filler aftercare for the first week. Ice on and off for the first day, sleep propped up, no gym, sauna or hot yoga for 48 hours, no pressing or massaging unless I asked you to, and keep the water up. Save the post on Instagram.</t>
+        </is>
+      </c>
+      <c r="F66" s="45" t="n">
+        <v>231</v>
+      </c>
+      <c r="G66" s="46" t="inlineStr">
+        <is>
+          <t>Your first week after lip filler, in the order it matters.
+First 48 hours: ice on and off, sleep propped up on an extra pillow, and skip the gym, sauna and hot yoga because heat and blood flow both make swelling worse. Do not press, pinch or massage the lips unless I have specifically told you to. No dental work, and hold off on flying if you can.
+Drink more water than usual. Hyaluronic acid draws water, and dehydrated lips feel tighter and look flatter.
+After 48 hours you are essentially back to normal. Small lumps in the first week are common and usually resolve on their own, but message me rather than sitting and worrying about it. Every client at the Oakville studio leaves with this in writing and my number. Save it from Instagram.</t>
+        </is>
+      </c>
+      <c r="H66" s="45" t="n">
+        <v>748</v>
+      </c>
+      <c r="I66" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J66" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K66" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-22-the-first-week.jpg</t>
+        </is>
+      </c>
+      <c r="L66" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M66" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N66" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-22-the-first-week.jpg")</f>
+        <v/>
+      </c>
+      <c r="O66" s="47" t="inlineStr">
+        <is>
+          <t>Soheil Kmp / Unsplash</t>
+        </is>
+      </c>
+      <c r="P66" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q66" s="46" t="inlineStr"/>
+    </row>
+    <row r="67" ht="132" customHeight="1" s="14">
+      <c r="A67" s="51" t="n">
+        <v>46318</v>
+      </c>
+      <c r="B67" s="45" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C67" s="45" t="inlineStr">
+        <is>
+          <t>IG: Aftercare Essentials</t>
+        </is>
+      </c>
+      <c r="D67" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E67" s="46" t="inlineStr">
+        <is>
+          <t>The whole filler aftercare list on one card. Ice, water, an extra pillow, no heat or hard exercise for 48 hours, no pressing at it, and no judging the result before two weeks. Save it to your phone. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F67" s="45" t="n">
+        <v>212</v>
+      </c>
+      <c r="G67" s="46" t="inlineStr">
+        <is>
+          <t>The entire filler aftercare list, on one card, because it really is short.
+Ice on and off for the first day. Water, more than you think. An extra pillow for two nights. No gym, sauna or hot yoga for 48 hours. No pressing, pinching or massaging the area. No judging the result until two weeks, which is the rule people break most.
+That is the list. Everything else you have read online is either a variation on those six or somebody selling you something.
+Every client at the Oakville studio leaves with this in writing and a way to reach me directly, because the reassuring answer at 9pm on day two is worth more than any leaflet. Save the card from Instagram so it is on your phone when you need it.</t>
+        </is>
+      </c>
+      <c r="H67" s="45" t="n">
+        <v>703</v>
+      </c>
+      <c r="I67" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J67" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K67" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-23-aftercare-essentials.jpg</t>
+        </is>
+      </c>
+      <c r="L67" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M67" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N67" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-23-aftercare-essentials.jpg")</f>
+        <v/>
+      </c>
+      <c r="O67" s="47" t="inlineStr">
+        <is>
+          <t>Rosa Rafael / Unsplash</t>
+        </is>
+      </c>
+      <c r="P67" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q67" s="46" t="inlineStr"/>
+    </row>
+    <row r="68" ht="132" customHeight="1" s="14">
+      <c r="A68" s="51" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B68" s="45" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C68" s="45" t="inlineStr">
+        <is>
+          <t>IG: Client Words: The Lip Glow-Up</t>
+        </is>
+      </c>
+      <c r="D68" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E68" s="46" t="inlineStr">
+        <is>
+          <t>In her words, shared with consent: she wanted lips that looked like hers on a good day, and nobody at work has asked what she had done. That is the brief, met. Her result is on Instagram beside it.</t>
+        </is>
+      </c>
+      <c r="F68" s="45" t="n">
+        <v>197</v>
+      </c>
+      <c r="G68" s="46" t="inlineStr">
+        <is>
+          <t>Her words, not mine, shared with her written consent.
+What she asked for was lips that looked like hers on a good day. Not bigger, not a shape she had saved from someone else. She had talked herself out of it twice, both times because of results she had seen on other people and did not want.
+We used less than one syringe, in a single appointment, and reviewed at two weeks.
+The line from her review that I keep thinking about: nobody at work has asked what she had done, and two people have asked if she has been sleeping better. That is the brief, met exactly. Her result is posted beside her words on Instagram, with permission. Lip filler consultations in Oakville are booked from there.</t>
+        </is>
+      </c>
+      <c r="H68" s="45" t="n">
+        <v>695</v>
+      </c>
+      <c r="I68" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J68" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K68" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-24-client-words-lips.jpg</t>
+        </is>
+      </c>
+      <c r="L68" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M68" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N68" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-24-client-words-lips.jpg")</f>
+        <v/>
+      </c>
+      <c r="O68" s="47" t="inlineStr">
+        <is>
+          <t>Elist Nguyen / Unsplash</t>
+        </is>
+      </c>
+      <c r="P68" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q68" s="46" t="inlineStr"/>
+    </row>
+    <row r="69" ht="132" customHeight="1" s="14">
+      <c r="A69" s="50" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B69" s="41" t="inlineStr">
+        <is>
+          <t>Sun</t>
+        </is>
+      </c>
+      <c r="C69" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D69" s="41" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E69" s="42" t="inlineStr">
+        <is>
+          <t>Booking is straightforward. Send a message on Instagram with what is bothering you and roughly when suits, and we start with a consult. Evenings available. Appointment only, at 3060 Preserve Dr, Oakville, with free parking at the door.</t>
+        </is>
+      </c>
+      <c r="F69" s="41" t="n">
+        <v>235</v>
+      </c>
+      <c r="G69" s="42" t="inlineStr">
+        <is>
+          <t>Booking at the Oakville studio is straightforward, and it starts with a conversation.
+Send a message on Instagram with what is bothering you and roughly when suits. You do not need to know which treatment you want, and you do not need the vocabulary. Describing it in your own words is genuinely enough, and often more useful.
+Every new client starts with a consult, which can be the same visit as treatment if you are a clear candidate and comfortable going ahead.
+We are appointment only at 3060 Preserve Dr, with free parking at the door and evening slots for people coming after work. Clients travel in from Burlington, Milton and Mississauga. Botox, lip filler, cheek filler and jawline, all injected by a nurse practitioner.</t>
+        </is>
+      </c>
+      <c r="H69" s="41" t="n">
+        <v>733</v>
+      </c>
+      <c r="I69" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J69" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K69" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-25-how-to-book-filler.jpg</t>
+        </is>
+      </c>
+      <c r="L69" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M69" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N69" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-25-how-to-book-filler.jpg")</f>
+        <v/>
+      </c>
+      <c r="O69" s="43" t="inlineStr">
+        <is>
+          <t>Look Studio / Unsplash</t>
+        </is>
+      </c>
+      <c r="P69" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q69" s="42" t="inlineStr"/>
+    </row>
+    <row r="70" ht="132" customHeight="1" s="14">
+      <c r="A70" s="51" t="n">
+        <v>46321</v>
+      </c>
+      <c r="B70" s="45" t="inlineStr">
+        <is>
+          <t>Mon</t>
+        </is>
+      </c>
+      <c r="C70" s="45" t="inlineStr">
+        <is>
+          <t>IG: 5 Filler Lies You Still Believe</t>
+        </is>
+      </c>
+      <c r="D70" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E70" s="46" t="inlineStr">
+        <is>
+          <t>Five filler lies, taken apart. It does not migrate on its own, it does not stretch your skin, it is not permanent, you are not committed for life, and one syringe is not a dramatic change. Every one of them has a real answer. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F70" s="45" t="n">
+        <v>239</v>
+      </c>
+      <c r="G70" s="46" t="inlineStr">
+        <is>
+          <t>Five things people still believe about filler, and what is actually true.
+It migrates on its own. It does not. Migration is overfilling or misplacement, and it is a technique problem, not a property of the product. It stretches your skin permanently. There is no good evidence for that at the volumes used properly. It is permanent. Hyaluronic acid filler is not, and it can be dissolved on purpose.
+Once you start you cannot stop. You can stop whenever you like, and your face returns to where it would have been.
+And the fifth, which is the most expensive one: that one syringe is a dramatic change. It is about a fifth of a teaspoon. All five taken apart properly on Instagram, or ask me directly at a consult in Oakville.</t>
+        </is>
+      </c>
+      <c r="H70" s="45" t="n">
+        <v>728</v>
+      </c>
+      <c r="I70" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J70" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K70" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-26-five-filler-lies.jpg</t>
+        </is>
+      </c>
+      <c r="L70" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M70" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N70" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-26-five-filler-lies.jpg")</f>
+        <v/>
+      </c>
+      <c r="O70" s="47" t="inlineStr">
+        <is>
+          <t>karelys Ruiz / Unsplash</t>
+        </is>
+      </c>
+      <c r="P70" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q70" s="46" t="inlineStr"/>
+    </row>
+    <row r="71" ht="132" customHeight="1" s="14">
+      <c r="A71" s="51" t="n">
+        <v>46322</v>
+      </c>
+      <c r="B71" s="45" t="inlineStr">
+        <is>
+          <t>Tue</t>
+        </is>
+      </c>
+      <c r="C71" s="45" t="inlineStr">
+        <is>
+          <t>IG: Myth vs Truth: Filler Edition</t>
+        </is>
+      </c>
+      <c r="D71" s="45" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="E71" s="46" t="inlineStr">
+        <is>
+          <t>Myth versus truth, filler edition. Six claims side by side, with the real answer next to each one. If you have been putting off asking because of something you read, one of these is probably it. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F71" s="45" t="n">
+        <v>208</v>
+      </c>
+      <c r="G71" s="46" t="inlineStr">
+        <is>
+          <t>Myth on one side, truth on the other, six of them.
+These are the six I hear most often at consults in Oakville, and they have a pattern. Every one of them started with somebody seeing a bad result and concluding that the treatment does that, rather than that the injector did that. Bad filler is loud and visible. Good filler is invisible by design, so it never gets counted.
+That asymmetry is the whole reason this misinformation survives.
+If you have been putting off asking a question because of something you read, there is a decent chance it is on this card with the real answer beside it. And if it is not, message me and I will answer it directly rather than sending you a leaflet. The card is on Instagram.</t>
+        </is>
+      </c>
+      <c r="H71" s="45" t="n">
+        <v>717</v>
+      </c>
+      <c r="I71" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J71" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K71" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-27-myth-vs-truth-filler.jpg</t>
+        </is>
+      </c>
+      <c r="L71" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M71" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N71" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-27-myth-vs-truth-filler.jpg")</f>
+        <v/>
+      </c>
+      <c r="O71" s="47" t="inlineStr">
+        <is>
+          <t>Ionela Mat / Unsplash</t>
+        </is>
+      </c>
+      <c r="P71" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q71" s="46" t="inlineStr"/>
+    </row>
+    <row r="72" ht="132" customHeight="1" s="14">
+      <c r="A72" s="50" t="n">
+        <v>46323</v>
+      </c>
+      <c r="B72" s="41" t="inlineStr">
+        <is>
+          <t>Wed</t>
+        </is>
+      </c>
+      <c r="C72" s="41" t="inlineStr">
+        <is>
+          <t>GBP only</t>
+        </is>
+      </c>
+      <c r="D72" s="41" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E72" s="42" t="inlineStr">
+        <is>
+          <t>How filler is priced here. Per syringe, quoted at your consult once we know the area and the amount, and half a syringe is priced as half. No package pressure and no product opened before you have agreed to the number.</t>
+        </is>
+      </c>
+      <c r="F72" s="41" t="n">
+        <v>218</v>
+      </c>
+      <c r="G72" s="42" t="inlineStr">
+        <is>
+          <t>Filler is priced per syringe, and you get the number before anything is opened.
+I do not post a price list, for the same reason I do not post one for Botox. The honest figure depends on the area, how much it actually needs and whether we are starting fresh or working alongside existing product, and a number posted without that context is either a lure or a guess.
+What you get instead: a quote at your consult, in writing, for the plan we agreed on. Half a syringe is priced as half.
+There are no packages to commit to and no pressure to book a series at the Oakville studio. If the plan is one syringe and a review, that is what you pay for. Ask at the consult and you will get a straight number.</t>
+        </is>
+      </c>
+      <c r="H72" s="41" t="n">
+        <v>702</v>
+      </c>
+      <c r="I72" s="41" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J72" s="43" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K72" s="41" t="inlineStr">
+        <is>
+          <t>2026-10-28-priced-by-the-syringe.jpg</t>
+        </is>
+      </c>
+      <c r="L72" s="43" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M72" s="43" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N72" s="41">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-28-priced-by-the-syringe.jpg")</f>
+        <v/>
+      </c>
+      <c r="O72" s="43" t="inlineStr">
+        <is>
+          <t>Masum Rahimi / Unsplash</t>
+        </is>
+      </c>
+      <c r="P72" s="41" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q72" s="42" t="inlineStr"/>
+    </row>
+    <row r="73" ht="132" customHeight="1" s="14">
+      <c r="A73" s="51" t="n">
+        <v>46324</v>
+      </c>
+      <c r="B73" s="45" t="inlineStr">
+        <is>
+          <t>Thu</t>
+        </is>
+      </c>
+      <c r="C73" s="45" t="inlineStr">
+        <is>
+          <t>IG: Facial Balancing: Why We Treat Faces, Not Lines</t>
+        </is>
+      </c>
+      <c r="D73" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E73" s="46" t="inlineStr">
+        <is>
+          <t>Why I treat faces and not lines. Chasing each line as it appears is how people end up overfilled and still unhappy, because the line was a symptom of lost support somewhere else. Fix the structure and the line softens. On Instagram.</t>
+        </is>
+      </c>
+      <c r="F73" s="45" t="n">
+        <v>232</v>
+      </c>
+      <c r="G73" s="46" t="inlineStr">
+        <is>
+          <t>Treating lines one at a time is how faces end up overfilled.
+A line is usually a symptom. The fold at the side of the mouth is the clearest example, since most of the time it is not a lack of volume at the fold, it is a lack of support above it that let the tissue settle. Fill the fold directly and you get a heavy, obvious result that still does not look right, and you will be back to fill it again.
+Support the structure and the line softens on its own, using less product in a place you were not looking at.
+This is the difference between an assessment and an order form. At the Oakville studio the consult starts with your whole face regardless of which line brought you in. The full explanation is on Instagram.</t>
+        </is>
+      </c>
+      <c r="H73" s="45" t="n">
+        <v>721</v>
+      </c>
+      <c r="I73" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J73" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K73" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-29-faces-not-lines.jpg</t>
+        </is>
+      </c>
+      <c r="L73" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M73" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N73" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-29-faces-not-lines.jpg")</f>
+        <v/>
+      </c>
+      <c r="O73" s="47" t="inlineStr">
+        <is>
+          <t>Elist Nguyen / Unsplash</t>
+        </is>
+      </c>
+      <c r="P73" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q73" s="46" t="inlineStr"/>
+    </row>
+    <row r="74" ht="132" customHeight="1" s="14">
+      <c r="A74" s="51" t="n">
+        <v>46325</v>
+      </c>
+      <c r="B74" s="45" t="inlineStr">
+        <is>
+          <t>Fri</t>
+        </is>
+      </c>
+      <c r="C74" s="45" t="inlineStr">
+        <is>
+          <t>IG: One Syringe. Balanced Lips.</t>
+        </is>
+      </c>
+      <c r="D74" s="45" t="inlineStr">
+        <is>
+          <t>Trust &amp; Proof</t>
+        </is>
+      </c>
+      <c r="E74" s="46" t="inlineStr">
+        <is>
+          <t>One syringe, one appointment, photographed two weeks apart in the same light. The upper lip was short against the lower, so the work was ratio rather than volume. Shared with client consent on Instagram.</t>
+        </is>
+      </c>
+      <c r="F74" s="45" t="n">
+        <v>203</v>
+      </c>
+      <c r="G74" s="46" t="inlineStr">
+        <is>
+          <t>One syringe, one appointment, and the photos are two weeks apart in the same light.
+The brief was balance rather than size. Her upper lip sat short against the lower, which made the whole mouth read slightly downturned in photos, and it was bothering her more in pictures than in the mirror. The work was ratio: height in the upper lip, support at the corners, nothing added for the sake of volume.
+Same lighting, same angle, no filter and no smoothing on either frame.
+If you look at these and think the change is subtle, that is the correct reaction and the reason she is happy with it. Shared with her written consent, on Instagram. Lip filler consultations in Oakville are booked from there, and half syringes are a real option.</t>
+        </is>
+      </c>
+      <c r="H74" s="45" t="n">
+        <v>735</v>
+      </c>
+      <c r="I74" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J74" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K74" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-30-one-syringe-balanced-lips.jpg</t>
+        </is>
+      </c>
+      <c r="L74" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M74" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N74" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-30-one-syringe-balanced-lips.jpg")</f>
+        <v/>
+      </c>
+      <c r="O74" s="47" t="inlineStr">
+        <is>
+          <t>Vitaliy Shevchenko / Unsplash</t>
+        </is>
+      </c>
+      <c r="P74" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q74" s="46" t="inlineStr"/>
+    </row>
+    <row r="75" ht="132" customHeight="1" s="14">
+      <c r="A75" s="51" t="n">
+        <v>46326</v>
+      </c>
+      <c r="B75" s="45" t="inlineStr">
+        <is>
+          <t>Sat</t>
+        </is>
+      </c>
+      <c r="C75" s="45" t="inlineStr">
+        <is>
+          <t>IG: Ask Anything: Filler Edition</t>
+        </is>
+      </c>
+      <c r="D75" s="45" t="inlineStr">
+        <is>
+          <t>Personality &amp; BTS</t>
+        </is>
+      </c>
+      <c r="E75" s="46" t="inlineStr">
+        <is>
+          <t>The question box is open all weekend, filler edition. Anonymous, and I answer the awkward ones first. Cost, pain, migration, dissolving, whether you are too young or too late. Ask on Instagram and I will answer this week.</t>
+        </is>
+      </c>
+      <c r="F75" s="45" t="n">
+        <v>221</v>
+      </c>
+      <c r="G75" s="46" t="inlineStr">
+        <is>
+          <t>The question box is open all weekend, filler edition. Ask me anything.
+It is anonymous, and I answer the awkward ones first because those are the ones stopping people from booking. Cost, pain, migration, dissolving, whether you are too young to start or too late to bother, what happens if you stop, what to do about work you had done somewhere else and do not like.
+October here has been a month about filler, and this is where it lands.
+Every answer goes up this week, and nothing gets skipped for being uncomfortable. If a question is better answered in person, I will say so rather than guessing at your face from a paragraph. Ask on Instagram, or book a consult at the Oakville studio and ask across the room.</t>
+        </is>
+      </c>
+      <c r="H75" s="45" t="n">
+        <v>717</v>
+      </c>
+      <c r="I75" s="45" t="inlineStr">
+        <is>
+          <t>Learn more</t>
+        </is>
+      </c>
+      <c r="J75" s="47" t="inlineStr">
+        <is>
+          <t>@luxury_beauty_aestheticz</t>
+        </is>
+      </c>
+      <c r="K75" s="45" t="inlineStr">
+        <is>
+          <t>2026-10-31-ask-anything-filler.jpg</t>
+        </is>
+      </c>
+      <c r="L75" s="47" t="inlineStr">
+        <is>
+          <t>Open folder</t>
+        </is>
+      </c>
+      <c r="M75" s="47" t="inlineStr">
+        <is>
+          <t>Open image</t>
+        </is>
+      </c>
+      <c r="N75" s="45">
+        <f>IMAGE("https://raw.githubusercontent.com/RepoKing23/InstagramCarousel/claude/med-spa-carousel-ideas-sim9wz/content/gbp/2026-10-31-ask-anything-filler.jpg")</f>
+        <v/>
+      </c>
+      <c r="O75" s="47" t="inlineStr">
+        <is>
+          <t>Alef Morais / Unsplash</t>
+        </is>
+      </c>
+      <c r="P75" s="45" t="inlineStr">
+        <is>
+          <t>Ready</t>
+        </is>
+      </c>
+      <c r="Q75" s="46" t="inlineStr"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -11835,6 +14283,130 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L44" r:id="rId170"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M44" r:id="rId171"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O44" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J45" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L45" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M45" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O45" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J46" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L46" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M46" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O46" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J47" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L47" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M47" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O47" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J48" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L48" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M48" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O48" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J49" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L49" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M49" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O49" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J50" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L50" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M50" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O50" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J51" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L51" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M51" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O51" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J52" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L52" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M52" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O52" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J53" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L53" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M53" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O53" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J54" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L54" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M54" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O54" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J55" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L55" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M55" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O55" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J56" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L56" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M56" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O56" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J57" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L57" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M57" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O57" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J58" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L58" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M58" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O58" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J59" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L59" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M59" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O59" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J60" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L60" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M60" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O60" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J61" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L61" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M61" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O61" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J62" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L62" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M62" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O62" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J63" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L63" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M63" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O63" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J64" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L64" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M64" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O64" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J65" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L65" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M65" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O65" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J66" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L66" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M66" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O66" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J67" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L67" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M67" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O67" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J68" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L68" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M68" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O68" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J69" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L69" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M69" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O69" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J70" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L70" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M70" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O70" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J71" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L71" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M71" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O71" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J72" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L72" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M72" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O72" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J73" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L73" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M73" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O73" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J74" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L74" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M74" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O74" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="J75" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="L75" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="M75" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="O75" r:id="rId296"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>